<commit_message>
Fill 40 more blank rows in the Tau-U prep sheet, figure over text
Second extraction round. Where the figure and the article text
disagree, values follow the figure (author's decision); each row's
note records what the text reports and where they differ. Phase
boundaries follow the figure's phase lines; 036-A D0356-D0358 are
set to baseline-vs-intervention comparisons accordingly.

Not filled: the three 17 Kern 2006 rows (scanned figure too blurry
to read reliably) and the 22 rows still waiting on a comparison
decision (022-A, Blair, Morrison, 017-A). D0290 keeps its baseline
trend blank to match the other 030-A post-training rows until that
question is decided. D0321/D0323 get a note only; values unchanged.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_015FN8gfsh3be5UpV8911V5L
</commit_message>
<xml_diff>
--- a/Tau-U计算前准备数据_完整版_中英对照_网格版_Claude补提取版.xlsx
+++ b/Tau-U计算前准备数据_完整版_中英对照_网格版_Claude补提取版.xlsx
@@ -7513,10 +7513,24 @@
           <t>Baseline（基线期） vs Maintenance（维持期）</t>
         </is>
       </c>
-      <c r="G79" s="22" t="n"/>
-      <c r="H79" s="23" t="n"/>
-      <c r="I79" s="22" t="n"/>
-      <c r="J79" s="23" t="n"/>
+      <c r="G79" s="22" t="inlineStr">
+        <is>
+          <t>0,0,0</t>
+        </is>
+      </c>
+      <c r="H79" s="23">
+        <f>IF(LEN(G79)=0,"",IF(ISNUMBER(SEARCH(",",G79)),LEN(SUBSTITUTE(G79,",","xx"))-LEN(G79)+1,1))</f>
+        <v/>
+      </c>
+      <c r="I79" s="22" t="inlineStr">
+        <is>
+          <t>83,83</t>
+        </is>
+      </c>
+      <c r="J79" s="23">
+        <f>IF(LEN(I79)=0,"",IF(ISNUMBER(SEARCH(",",I79)),LEN(SUBSTITUTE(I79,",","xx"))-LEN(I79)+1,1))</f>
+        <v/>
+      </c>
       <c r="K79" s="18" t="inlineStr">
         <is>
           <t>%</t>
@@ -7527,9 +7541,16 @@
           <t>升高改善</t>
         </is>
       </c>
-      <c r="M79" s="39" t="n"/>
-      <c r="N79" s="39" t="n"/>
-      <c r="O79" s="21" t="n"/>
+      <c r="M79" s="39" t="n">
+        <v>0</v>
+      </c>
+      <c r="N79" s="39" t="n">
+        <v>1</v>
+      </c>
+      <c r="O79" s="21">
+        <f>IF(AND(N79&lt;0.05,OR(AND(L79="升高改善",M79&gt;0),AND(L79="降低改善",M79&lt;0))),"校正","不校正")</f>
+        <v/>
+      </c>
       <c r="P79" s="18" t="inlineStr">
         <is>
           <t>Figure 1；PDF第8页，印刷页8；上方面板 Amber/Regina；实心方形（Child w/ ASD，独立接受游戏邀请的步骤）；实心三角形为 Typical Peer。</t>
@@ -7537,17 +7558,17 @@
       </c>
       <c r="Q79" s="18" t="inlineStr">
         <is>
-          <t>GPT</t>
+          <t>Claude</t>
         </is>
       </c>
       <c r="R79" s="24" t="inlineStr">
         <is>
-          <t>待审核</t>
+          <t>Claude补提取</t>
         </is>
       </c>
       <c r="S79" s="18" t="inlineStr">
         <is>
-          <t>待审核：维持阶段两个图示点与正文报告不一致，尚不能判定图或文字何者有误，需核实维持期数据。</t>
+          <t>Claude补提取（以图为准）：从PDF第8页内嵌原图（836×1403像素）逐像素检测实心方块（Child w/ ASD），按纵轴刻度（4像素/单位）换算；阶段线为PDF矢量叠加层，干预与维持分界位于第16、17次之间（三个面板共用）。图文不一致：维持期图上2个方块均为83%（第18、19次；与三角形部分重叠，按方块上缘推算），正文报告Regina维持75%。按图取值。维持期只有2点（&lt;3点规则待定）。</t>
         </is>
       </c>
     </row>
@@ -7756,10 +7777,24 @@
           <t>Baseline（基线期） vs VM（视频示范）</t>
         </is>
       </c>
-      <c r="G82" s="22" t="n"/>
-      <c r="H82" s="23" t="n"/>
-      <c r="I82" s="22" t="n"/>
-      <c r="J82" s="23" t="n"/>
+      <c r="G82" s="22" t="inlineStr">
+        <is>
+          <t>0,0,0,0,0</t>
+        </is>
+      </c>
+      <c r="H82" s="23">
+        <f>IF(LEN(G82)=0,"",IF(ISNUMBER(SEARCH(",",G82)),LEN(SUBSTITUTE(G82,",","xx"))-LEN(G82)+1,1))</f>
+        <v/>
+      </c>
+      <c r="I82" s="22" t="inlineStr">
+        <is>
+          <t>58,100,100,83</t>
+        </is>
+      </c>
+      <c r="J82" s="23">
+        <f>IF(LEN(I82)=0,"",IF(ISNUMBER(SEARCH(",",I82)),LEN(SUBSTITUTE(I82,",","xx"))-LEN(I82)+1,1))</f>
+        <v/>
+      </c>
       <c r="K82" s="18" t="inlineStr">
         <is>
           <t>%</t>
@@ -7770,9 +7805,16 @@
           <t>升高改善</t>
         </is>
       </c>
-      <c r="M82" s="39" t="n"/>
-      <c r="N82" s="39" t="n"/>
-      <c r="O82" s="21" t="n"/>
+      <c r="M82" s="39" t="n">
+        <v>0</v>
+      </c>
+      <c r="N82" s="39" t="n">
+        <v>1</v>
+      </c>
+      <c r="O82" s="21">
+        <f>IF(AND(N82&lt;0.05,OR(AND(L82="升高改善",M82&gt;0),AND(L82="降低改善",M82&lt;0))),"校正","不校正")</f>
+        <v/>
+      </c>
       <c r="P82" s="18" t="inlineStr">
         <is>
           <t>Figure 1；PDF第8页，印刷页8；下方面板 Milo/Xane；实心方形（Child w/ ASD，独立接受游戏邀请的步骤）；实心三角形为 Typical Peer。</t>
@@ -7780,17 +7822,17 @@
       </c>
       <c r="Q82" s="18" t="inlineStr">
         <is>
-          <t>GPT</t>
+          <t>Claude</t>
         </is>
       </c>
       <c r="R82" s="24" t="inlineStr">
         <is>
-          <t>待审核</t>
+          <t>Claude补提取</t>
         </is>
       </c>
       <c r="S82" s="18" t="inlineStr">
         <is>
-          <t>待审核：首个干预观察点的图示读值与正文描述不一致，需核实该点后确认完整干预序列。</t>
+          <t>Claude补提取（以图为准）：从PDF第8页内嵌原图（836×1403像素）逐像素检测实心方块（Child w/ ASD），按纵轴刻度（4像素/单位）换算；阶段线为PDF矢量叠加层，干预与维持分界位于第16、17次之间（三个面板共用）。基线5次探测（第1、2、3、7、11次）均为0。干预期按矢量阶段线为第12–15次4点：58,100,100,83。图文不一致：第1个干预点图上为58%（约为7/12步），正文写60%；第15次的83%按阶段线属于干预期，而正文说“维持83%”。按图取值。</t>
         </is>
       </c>
     </row>
@@ -7825,10 +7867,24 @@
           <t>Baseline（基线期） vs Maintenance（维持期）</t>
         </is>
       </c>
-      <c r="G83" s="22" t="n"/>
-      <c r="H83" s="23" t="n"/>
-      <c r="I83" s="22" t="n"/>
-      <c r="J83" s="23" t="n"/>
+      <c r="G83" s="22" t="inlineStr">
+        <is>
+          <t>0,0,0,0,0</t>
+        </is>
+      </c>
+      <c r="H83" s="23">
+        <f>IF(LEN(G83)=0,"",IF(ISNUMBER(SEARCH(",",G83)),LEN(SUBSTITUTE(G83,",","xx"))-LEN(G83)+1,1))</f>
+        <v/>
+      </c>
+      <c r="I83" s="22" t="inlineStr">
+        <is>
+          <t>92,100</t>
+        </is>
+      </c>
+      <c r="J83" s="23">
+        <f>IF(LEN(I83)=0,"",IF(ISNUMBER(SEARCH(",",I83)),LEN(SUBSTITUTE(I83,",","xx"))-LEN(I83)+1,1))</f>
+        <v/>
+      </c>
       <c r="K83" s="18" t="inlineStr">
         <is>
           <t>%</t>
@@ -7839,9 +7895,16 @@
           <t>升高改善</t>
         </is>
       </c>
-      <c r="M83" s="39" t="n"/>
-      <c r="N83" s="39" t="n"/>
-      <c r="O83" s="21" t="n"/>
+      <c r="M83" s="39" t="n">
+        <v>0</v>
+      </c>
+      <c r="N83" s="39" t="n">
+        <v>1</v>
+      </c>
+      <c r="O83" s="21">
+        <f>IF(AND(N83&lt;0.05,OR(AND(L83="升高改善",M83&gt;0),AND(L83="降低改善",M83&lt;0))),"校正","不校正")</f>
+        <v/>
+      </c>
       <c r="P83" s="18" t="inlineStr">
         <is>
           <t>Figure 1；PDF第8页，印刷页8；下方面板 Milo/Xane；实心方形（Child w/ ASD，独立接受游戏邀请的步骤）；实心三角形为 Typical Peer。</t>
@@ -7849,17 +7912,17 @@
       </c>
       <c r="Q83" s="18" t="inlineStr">
         <is>
-          <t>GPT</t>
+          <t>Claude</t>
         </is>
       </c>
       <c r="R83" s="24" t="inlineStr">
         <is>
-          <t>待审核</t>
+          <t>Claude补提取</t>
         </is>
       </c>
       <c r="S83" s="18" t="inlineStr">
         <is>
-          <t>待审核：维持阶段两个图示点与正文报告的水平不一致，需核实原始观察记录和维持期数值。</t>
+          <t>Claude补提取（以图为准）：从PDF第8页内嵌原图（836×1403像素）逐像素检测实心方块（Child w/ ASD），按纵轴刻度（4像素/单位）换算；阶段线为PDF矢量叠加层，干预与维持分界位于第16、17次之间（三个面板共用）。维持期按矢量阶段线为第18、19次：92,100（第18次方块与三角形重叠，按方块上缘推算）。图文不一致：正文报告Xane维持83%，图上维持期为92、100。按图取值。维持期只有2点（&lt;3点规则待定）。</t>
         </is>
       </c>
     </row>
@@ -14108,10 +14171,24 @@
           <t>Baseline（基线期） vs Intervention（干预期）</t>
         </is>
       </c>
-      <c r="G156" s="33" t="n"/>
-      <c r="H156" s="34" t="n"/>
-      <c r="I156" s="33" t="n"/>
-      <c r="J156" s="34" t="n"/>
+      <c r="G156" s="33" t="inlineStr">
+        <is>
+          <t>8.0,5.0,36.2,6.6,52.4,10.5</t>
+        </is>
+      </c>
+      <c r="H156" s="34">
+        <f>IF(LEN(G156)=0,"",IF(ISNUMBER(SEARCH(",",G156)),LEN(SUBSTITUTE(G156,",","xx"))-LEN(G156)+1,1))</f>
+        <v/>
+      </c>
+      <c r="I156" s="33" t="inlineStr">
+        <is>
+          <t>47.4,29.2,60.0,50.0,52.8,31.6,70.0,79.2</t>
+        </is>
+      </c>
+      <c r="J156" s="34">
+        <f>IF(LEN(I156)=0,"",IF(ISNUMBER(SEARCH(",",I156)),LEN(SUBSTITUTE(I156,",","xx"))-LEN(I156)+1,1))</f>
+        <v/>
+      </c>
       <c r="K156" s="13" t="inlineStr">
         <is>
           <t>%</t>
@@ -14122,9 +14199,16 @@
           <t>升高改善</t>
         </is>
       </c>
-      <c r="M156" s="38" t="n"/>
-      <c r="N156" s="38" t="n"/>
-      <c r="O156" s="16" t="n"/>
+      <c r="M156" s="38" t="n">
+        <v>0.3333333333333333</v>
+      </c>
+      <c r="N156" s="38" t="n">
+        <v>0.347558036741169</v>
+      </c>
+      <c r="O156" s="16">
+        <f>IF(AND(N156&lt;0.05,OR(AND(L156="升高改善",M156&gt;0),AND(L156="降低改善",M156&lt;0))),"校正","不校正")</f>
+        <v/>
+      </c>
       <c r="P156" s="13" t="inlineStr">
         <is>
           <t>Figure 1；PDF第7页／印刷第7页；第1（上）面板（James）；黑色实心圆、实线连接；灰三角为Intervention fidelity，排除。</t>
@@ -14132,17 +14216,17 @@
       </c>
       <c r="Q156" s="13" t="inlineStr">
         <is>
-          <t>GPT</t>
+          <t>Claude</t>
         </is>
       </c>
       <c r="R156" s="35" t="inlineStr">
         <is>
-          <t>待审核</t>
+          <t>Claude补提取</t>
         </is>
       </c>
       <c r="S156" s="13" t="inlineStr">
         <is>
-          <t>待审核：基线第11次观察的图示读值超出正文报告范围，图文最大值冲突，需核实该点。</t>
+          <t>Claude补提取（以图为准）：Figure为PDF矢量图，直接读取实心圆的PDF坐标，按各面板纵轴（0%至100%）线性换算，保留1位小数；同法复核GPT已填的Aaron、Edward、James离任务数据，结果一致。图文不一致：基线第5点（约第11次）图上为52.4%，超出正文范围5–36%；但含此点的基线均值19.8%与正文均值20%一致，说明正文范围有误。干预8点均值52.5%、范围29.2–79.2%，与正文53%（29–79%）一致。按图取值。</t>
         </is>
       </c>
     </row>
@@ -14177,10 +14261,24 @@
           <t>Baseline（基线期） vs Maintenance（维持期）</t>
         </is>
       </c>
-      <c r="G157" s="22" t="n"/>
-      <c r="H157" s="23" t="n"/>
-      <c r="I157" s="22" t="n"/>
-      <c r="J157" s="23" t="n"/>
+      <c r="G157" s="22" t="inlineStr">
+        <is>
+          <t>8.0,5.0,36.2,6.6,52.4,10.5</t>
+        </is>
+      </c>
+      <c r="H157" s="23">
+        <f>IF(LEN(G157)=0,"",IF(ISNUMBER(SEARCH(",",G157)),LEN(SUBSTITUTE(G157,",","xx"))-LEN(G157)+1,1))</f>
+        <v/>
+      </c>
+      <c r="I157" s="22" t="inlineStr">
+        <is>
+          <t>8.4</t>
+        </is>
+      </c>
+      <c r="J157" s="23">
+        <f>IF(LEN(I157)=0,"",IF(ISNUMBER(SEARCH(",",I157)),LEN(SUBSTITUTE(I157,",","xx"))-LEN(I157)+1,1))</f>
+        <v/>
+      </c>
       <c r="K157" s="18" t="inlineStr">
         <is>
           <t>%</t>
@@ -14191,9 +14289,16 @@
           <t>升高改善</t>
         </is>
       </c>
-      <c r="M157" s="39" t="n"/>
-      <c r="N157" s="39" t="n"/>
-      <c r="O157" s="21" t="n"/>
+      <c r="M157" s="39" t="n">
+        <v>0.3333333333333333</v>
+      </c>
+      <c r="N157" s="39" t="n">
+        <v>0.347558036741169</v>
+      </c>
+      <c r="O157" s="21">
+        <f>IF(AND(N157&lt;0.05,OR(AND(L157="升高改善",M157&gt;0),AND(L157="降低改善",M157&lt;0))),"校正","不校正")</f>
+        <v/>
+      </c>
       <c r="P157" s="18" t="inlineStr">
         <is>
           <t>Figure 1；PDF第7页／印刷第7页；第1（上）面板（James）；黑色实心圆、实线连接；维持为最右单点；灰三角为Intervention fidelity，排除。</t>
@@ -14201,17 +14306,17 @@
       </c>
       <c r="Q157" s="18" t="inlineStr">
         <is>
-          <t>GPT</t>
+          <t>Claude</t>
         </is>
       </c>
       <c r="R157" s="24" t="inlineStr">
         <is>
-          <t>待审核</t>
+          <t>Claude补提取</t>
         </is>
       </c>
       <c r="S157" s="18" t="inlineStr">
         <is>
-          <t>待审核：基线第11次观察的图示读值超出正文报告范围，图文最大值冲突，需核实该点。</t>
+          <t>Claude补提取（以图为准）：Figure为PDF矢量图，直接读取实心圆的PDF坐标，按各面板纵轴（0%至100%）线性换算，保留1位小数；同法复核GPT已填的Aaron、Edward、James离任务数据，结果一致。基线同D0155（基线第5点52.4%超出正文范围，见D0155）。维持探测1次8.4%，与正文8%一致。维持期只有1点（&lt;3点规则待定）。</t>
         </is>
       </c>
     </row>
@@ -14418,10 +14523,24 @@
           <t>Baseline（基线期） vs Intervention（干预期）</t>
         </is>
       </c>
-      <c r="G160" s="22" t="n"/>
-      <c r="H160" s="23" t="n"/>
-      <c r="I160" s="22" t="n"/>
-      <c r="J160" s="23" t="n"/>
+      <c r="G160" s="22" t="inlineStr">
+        <is>
+          <t>53.5,36.6,55.9,89.9,68.3</t>
+        </is>
+      </c>
+      <c r="H160" s="23">
+        <f>IF(LEN(G160)=0,"",IF(ISNUMBER(SEARCH(",",G160)),LEN(SUBSTITUTE(G160,",","xx"))-LEN(G160)+1,1))</f>
+        <v/>
+      </c>
+      <c r="I160" s="22" t="inlineStr">
+        <is>
+          <t>81.8,84.9,89.9,89.2</t>
+        </is>
+      </c>
+      <c r="J160" s="23">
+        <f>IF(LEN(I160)=0,"",IF(ISNUMBER(SEARCH(",",I160)),LEN(SUBSTITUTE(I160,",","xx"))-LEN(I160)+1,1))</f>
+        <v/>
+      </c>
       <c r="K160" s="18" t="inlineStr">
         <is>
           <t>%</t>
@@ -14432,9 +14551,16 @@
           <t>升高改善</t>
         </is>
       </c>
-      <c r="M160" s="39" t="n"/>
-      <c r="N160" s="39" t="n"/>
-      <c r="O160" s="21" t="n"/>
+      <c r="M160" s="39" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="N160" s="39" t="n">
+        <v>0.1416446902951368</v>
+      </c>
+      <c r="O160" s="21">
+        <f>IF(AND(N160&lt;0.05,OR(AND(L160="升高改善",M160&gt;0),AND(L160="降低改善",M160&lt;0))),"校正","不校正")</f>
+        <v/>
+      </c>
       <c r="P160" s="18" t="inlineStr">
         <is>
           <t>Figure 1；PDF第7页／印刷第7页；第4（下）面板（Sam）；黑色实心圆、实线连接；灰三角为Intervention fidelity，排除。</t>
@@ -14442,17 +14568,17 @@
       </c>
       <c r="Q160" s="18" t="inlineStr">
         <is>
-          <t>GPT</t>
+          <t>Claude</t>
         </is>
       </c>
       <c r="R160" s="24" t="inlineStr">
         <is>
-          <t>待审核</t>
+          <t>Claude补提取</t>
         </is>
       </c>
       <c r="S160" s="18" t="inlineStr">
         <is>
-          <t>待审核：干预第39次观察的图示读值低于正文报告范围，图文最小值冲突，需核实该点。</t>
+          <t>Claude补提取（以图为准）：Figure为PDF矢量图，直接读取实心圆的PDF坐标，按各面板纵轴（0%至100%）线性换算，保留1位小数；同法复核GPT已填的Aaron、Edward、James离任务数据，结果一致。基线5点均值60.8%、范围36.6–89.9%，与正文61%（37–90%）一致。图文不一致：干预第1点（第39次）图上为81.8%，低于正文范围85–90%；干预均值86.5%与正文86%一致。按图取值。</t>
         </is>
       </c>
     </row>
@@ -14745,10 +14871,24 @@
           <t>Baseline（基线期） vs Intervention（干预期）</t>
         </is>
       </c>
-      <c r="G164" s="22" t="n"/>
-      <c r="H164" s="23" t="n"/>
-      <c r="I164" s="22" t="n"/>
-      <c r="J164" s="23" t="n"/>
+      <c r="G164" s="22" t="inlineStr">
+        <is>
+          <t>0.0,81.0,43.5,70.0,80.0,91.3</t>
+        </is>
+      </c>
+      <c r="H164" s="23">
+        <f>IF(LEN(G164)=0,"",IF(ISNUMBER(SEARCH(",",G164)),LEN(SUBSTITUTE(G164,",","xx"))-LEN(G164)+1,1))</f>
+        <v/>
+      </c>
+      <c r="I164" s="22" t="inlineStr">
+        <is>
+          <t>43.6,65.2,60.0,40.6</t>
+        </is>
+      </c>
+      <c r="J164" s="23">
+        <f>IF(LEN(I164)=0,"",IF(ISNUMBER(SEARCH(",",I164)),LEN(SUBSTITUTE(I164,",","xx"))-LEN(I164)+1,1))</f>
+        <v/>
+      </c>
       <c r="K164" s="18" t="inlineStr">
         <is>
           <t>%</t>
@@ -14759,9 +14899,16 @@
           <t>降低改善</t>
         </is>
       </c>
-      <c r="M164" s="39" t="n"/>
-      <c r="N164" s="39" t="n"/>
-      <c r="O164" s="21" t="n"/>
+      <c r="M164" s="39" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="N164" s="39" t="n">
+        <v>0.09087393998624903</v>
+      </c>
+      <c r="O164" s="21">
+        <f>IF(AND(N164&lt;0.05,OR(AND(L164="升高改善",M164&gt;0),AND(L164="降低改善",M164&lt;0))),"校正","不校正")</f>
+        <v/>
+      </c>
       <c r="P164" s="18" t="inlineStr">
         <is>
           <t>Figure 2；PDF第8页／印刷第8页；第3面板（Edward）；黑色实心圆、实线连接。</t>
@@ -14769,17 +14916,17 @@
       </c>
       <c r="Q164" s="18" t="inlineStr">
         <is>
-          <t>GPT</t>
+          <t>Claude</t>
         </is>
       </c>
       <c r="R164" s="24" t="inlineStr">
         <is>
-          <t>待审核</t>
+          <t>Claude补提取</t>
         </is>
       </c>
       <c r="S164" s="18" t="inlineStr">
         <is>
-          <t>待审核：基线及干预图示均值与正文不符，且正文干预均值不在其所报范围内，尚无法定位具体错误。</t>
+          <t>Claude补提取（以图为准）：Figure为PDF矢量图，直接读取实心圆的PDF坐标，按各面板纵轴（0%至100%）线性换算，保留1位小数；同法复核GPT已填的Aaron、Edward、James离任务数据，结果一致。读Figure 2（PDF第8页）。图文不一致：基线均值图上61.0%、正文65%（范围0–92%与图一致）；干预均值图上52.4%，正文写22%，但正文给的范围41–65%与图一致，正文均值22%本身不在其范围内，应为正文笔误。按图取值。</t>
         </is>
       </c>
     </row>
@@ -14814,10 +14961,24 @@
           <t>Baseline（基线期） vs Intervention（干预期）</t>
         </is>
       </c>
-      <c r="G165" s="22" t="n"/>
-      <c r="H165" s="23" t="n"/>
-      <c r="I165" s="22" t="n"/>
-      <c r="J165" s="23" t="n"/>
+      <c r="G165" s="22" t="inlineStr">
+        <is>
+          <t>16.0,51.6,31.9,6.6,24.9</t>
+        </is>
+      </c>
+      <c r="H165" s="23">
+        <f>IF(LEN(G165)=0,"",IF(ISNUMBER(SEARCH(",",G165)),LEN(SUBSTITUTE(G165,",","xx"))-LEN(G165)+1,1))</f>
+        <v/>
+      </c>
+      <c r="I165" s="22" t="inlineStr">
+        <is>
+          <t>38.9,22.5,7.4,29.7</t>
+        </is>
+      </c>
+      <c r="J165" s="23">
+        <f>IF(LEN(I165)=0,"",IF(ISNUMBER(SEARCH(",",I165)),LEN(SUBSTITUTE(I165,",","xx"))-LEN(I165)+1,1))</f>
+        <v/>
+      </c>
       <c r="K165" s="18" t="inlineStr">
         <is>
           <t>%</t>
@@ -14828,9 +14989,16 @@
           <t>降低改善</t>
         </is>
       </c>
-      <c r="M165" s="39" t="n"/>
-      <c r="N165" s="39" t="n"/>
-      <c r="O165" s="21" t="n"/>
+      <c r="M165" s="39" t="n">
+        <v>-0.2</v>
+      </c>
+      <c r="N165" s="39" t="n">
+        <v>0.624206114766406</v>
+      </c>
+      <c r="O165" s="21">
+        <f>IF(AND(N165&lt;0.05,OR(AND(L165="升高改善",M165&gt;0),AND(L165="降低改善",M165&lt;0))),"校正","不校正")</f>
+        <v/>
+      </c>
       <c r="P165" s="18" t="inlineStr">
         <is>
           <t>Figure 2；PDF第8页／印刷第8页；第4（下）面板（Sam）；黑色实心圆、实线连接。</t>
@@ -14838,17 +15006,17 @@
       </c>
       <c r="Q165" s="18" t="inlineStr">
         <is>
-          <t>GPT</t>
+          <t>Claude</t>
         </is>
       </c>
       <c r="R165" s="24" t="inlineStr">
         <is>
-          <t>待审核</t>
+          <t>Claude补提取</t>
         </is>
       </c>
       <c r="S165" s="18" t="inlineStr">
         <is>
-          <t>待审核：基线第22次观察的图示读值超出正文报告范围，图文最大值冲突，需核实该点。</t>
+          <t>Claude补提取（以图为准）：Figure为PDF矢量图，直接读取实心圆的PDF坐标，按各面板纵轴（0%至100%）线性换算，保留1位小数；同法复核GPT已填的Aaron、Edward、James离任务数据，结果一致。读Figure 2（PDF第8页）。图文不一致：基线第2点（第22次）图上为51.6%，超出正文范围7–32%；但含此点的基线均值26.2%与正文26%一致。干预4点均值24.6%、范围7.4–38.9%，与正文25%（7.5–39%）一致。按图取值。</t>
         </is>
       </c>
     </row>
@@ -15227,10 +15395,24 @@
           <t>Baseline（基线期） vs Intervention- PMI（同伴介入干预期）</t>
         </is>
       </c>
-      <c r="G170" s="33" t="n"/>
-      <c r="H170" s="34" t="n"/>
-      <c r="I170" s="33" t="n"/>
-      <c r="J170" s="34" t="n"/>
+      <c r="G170" s="33" t="inlineStr">
+        <is>
+          <t>6,7,7,8</t>
+        </is>
+      </c>
+      <c r="H170" s="34">
+        <f>IF(LEN(G170)=0,"",IF(ISNUMBER(SEARCH(",",G170)),LEN(SUBSTITUTE(G170,",","xx"))-LEN(G170)+1,1))</f>
+        <v/>
+      </c>
+      <c r="I170" s="33" t="inlineStr">
+        <is>
+          <t>4,5,3,2,2,3,2,2</t>
+        </is>
+      </c>
+      <c r="J170" s="34">
+        <f>IF(LEN(I170)=0,"",IF(ISNUMBER(SEARCH(",",I170)),LEN(SUBSTITUTE(I170,",","xx"))-LEN(I170)+1,1))</f>
+        <v/>
+      </c>
       <c r="K170" s="3" t="inlineStr">
         <is>
           <t>错误次数</t>
@@ -15241,9 +15423,16 @@
           <t>降低改善</t>
         </is>
       </c>
-      <c r="M170" s="38" t="n"/>
-      <c r="N170" s="38" t="n"/>
-      <c r="O170" s="16" t="n"/>
+      <c r="M170" s="38" t="n">
+        <v>0.9128709291752769</v>
+      </c>
+      <c r="N170" s="38" t="n">
+        <v>0.07095149242730563</v>
+      </c>
+      <c r="O170" s="16">
+        <f>IF(AND(N170&lt;0.05,OR(AND(L170="升高改善",M170&gt;0),AND(L170="降低改善",M170&lt;0))),"校正","不校正")</f>
+        <v/>
+      </c>
       <c r="P170" s="3" t="inlineStr">
         <is>
           <t>Figure 1；PDF第7页，印刷页7；上方面板 Subject-Verb Agreement；实心圆形；纵轴 Number of errors。</t>
@@ -15251,17 +15440,17 @@
       </c>
       <c r="Q170" s="3" t="inlineStr">
         <is>
-          <t>GPT</t>
+          <t>Claude</t>
         </is>
       </c>
       <c r="R170" s="35" t="inlineStr">
         <is>
-          <t>待审核</t>
+          <t>Claude补提取</t>
         </is>
       </c>
       <c r="S170" s="3" t="inlineStr">
         <is>
-          <t>待审核：干预图有8个观察点，正文同时写8天和5次，观测点数及各次记录的对应关系需核实。</t>
+          <t>Claude补提取（以图为准）：读PDF第7页Figure 1（300 dpi渲染），逐像素检测实心圆，按纵轴刻度标签换算，读数均为整数。图上干预期8点，均值2.875，与正文/表3均值2.9、范围2–5一致；正文“8天（5次40分钟课）”的次数说法与点数不符，按图取8点。基线与D0170相同。</t>
         </is>
       </c>
     </row>
@@ -15562,10 +15751,24 @@
           <t>Baseline（基线期） vs Intervention- PMI（同伴介入干预期）</t>
         </is>
       </c>
-      <c r="G174" s="22" t="n"/>
-      <c r="H174" s="23" t="n"/>
-      <c r="I174" s="22" t="n"/>
-      <c r="J174" s="23" t="n"/>
+      <c r="G174" s="22" t="inlineStr">
+        <is>
+          <t>5,4,6,6,5,6,8,7,6,7,7,6,6,8,7,5,6</t>
+        </is>
+      </c>
+      <c r="H174" s="23">
+        <f>IF(LEN(G174)=0,"",IF(ISNUMBER(SEARCH(",",G174)),LEN(SUBSTITUTE(G174,",","xx"))-LEN(G174)+1,1))</f>
+        <v/>
+      </c>
+      <c r="I174" s="22" t="inlineStr">
+        <is>
+          <t>6,4,3,3,2,3,2</t>
+        </is>
+      </c>
+      <c r="J174" s="23">
+        <f>IF(LEN(I174)=0,"",IF(ISNUMBER(SEARCH(",",I174)),LEN(SUBSTITUTE(I174,",","xx"))-LEN(I174)+1,1))</f>
+        <v/>
+      </c>
       <c r="K174" s="8" t="inlineStr">
         <is>
           <t>错误次数</t>
@@ -15576,9 +15779,16 @@
           <t>降低改善</t>
         </is>
       </c>
-      <c r="M174" s="39" t="n"/>
-      <c r="N174" s="39" t="n"/>
-      <c r="O174" s="21" t="n"/>
+      <c r="M174" s="39" t="n">
+        <v>0.2761530448893886</v>
+      </c>
+      <c r="N174" s="39" t="n">
+        <v>0.1523786670550124</v>
+      </c>
+      <c r="O174" s="21">
+        <f>IF(AND(N174&lt;0.05,OR(AND(L174="升高改善",M174&gt;0),AND(L174="降低改善",M174&lt;0))),"校正","不校正")</f>
+        <v/>
+      </c>
       <c r="P174" s="8" t="inlineStr">
         <is>
           <t>Figure 1；PDF第7页，印刷页7；下方面板 Punctuation；实心圆形；纵轴 Number of errors。</t>
@@ -15586,17 +15796,17 @@
       </c>
       <c r="Q174" s="8" t="inlineStr">
         <is>
-          <t>GPT</t>
+          <t>Claude</t>
         </is>
       </c>
       <c r="R174" s="24" t="inlineStr">
         <is>
-          <t>待审核</t>
+          <t>Claude补提取</t>
         </is>
       </c>
       <c r="S174" s="8" t="inlineStr">
         <is>
-          <t>待审核：干预图有7个观察点，正文同时写7天和8次，观测点数及各次记录的对应关系需核实。</t>
+          <t>Claude补提取（以图为准）：读PDF第7页Figure 1（300 dpi渲染），逐像素检测实心圆，按纵轴刻度标签换算，读数均为整数。图上干预期7点，均值3.29，范围2–6；正文/表3报告均值3.2、范围2–6，正文写“7天8次”。点数与均值和正文略有出入，无法定位，按图取7点。基线与D0174相同。</t>
         </is>
       </c>
     </row>
@@ -17805,10 +18015,24 @@
           <t>Baseline（基线期） vs Intervention（干预期）</t>
         </is>
       </c>
-      <c r="G200" s="22" t="n"/>
-      <c r="H200" s="23" t="n"/>
-      <c r="I200" s="22" t="n"/>
-      <c r="J200" s="23" t="n"/>
+      <c r="G200" s="22" t="inlineStr">
+        <is>
+          <t>0,0,0,0,0,0,0,0,0</t>
+        </is>
+      </c>
+      <c r="H200" s="23">
+        <f>IF(LEN(G200)=0,"",IF(ISNUMBER(SEARCH(",",G200)),LEN(SUBSTITUTE(G200,",","xx"))-LEN(G200)+1,1))</f>
+        <v/>
+      </c>
+      <c r="I200" s="22" t="inlineStr">
+        <is>
+          <t>100,26.1,38.1,100</t>
+        </is>
+      </c>
+      <c r="J200" s="23">
+        <f>IF(LEN(I200)=0,"",IF(ISNUMBER(SEARCH(",",I200)),LEN(SUBSTITUTE(I200,",","xx"))-LEN(I200)+1,1))</f>
+        <v/>
+      </c>
       <c r="K200" s="18" t="inlineStr">
         <is>
           <t>%</t>
@@ -17819,9 +18043,16 @@
           <t>升高改善</t>
         </is>
       </c>
-      <c r="M200" s="39" t="n"/>
-      <c r="N200" s="39" t="n"/>
-      <c r="O200" s="21" t="n"/>
+      <c r="M200" s="39" t="n">
+        <v>0</v>
+      </c>
+      <c r="N200" s="39" t="n">
+        <v>1</v>
+      </c>
+      <c r="O200" s="21">
+        <f>IF(AND(N200&lt;0.05,OR(AND(L200="升高改善",M200&gt;0),AND(L200="降低改善",M200&lt;0))),"校正","不校正")</f>
+        <v/>
+      </c>
       <c r="P200" s="18" t="inlineStr">
         <is>
           <t>Figure 1；PDF第6页，印刷页76；下方面板 Dyad 3（Robert）；实心黑色菱形、左纵轴（Target child responses）；空心圆形及右纵轴为同伴发起。</t>
@@ -17829,17 +18060,17 @@
       </c>
       <c r="Q200" s="18" t="inlineStr">
         <is>
-          <t>GPT</t>
+          <t>Claude</t>
         </is>
       </c>
       <c r="R200" s="24" t="inlineStr">
         <is>
-          <t>待审核</t>
+          <t>Claude补提取</t>
         </is>
       </c>
       <c r="S200" s="18" t="inlineStr">
         <is>
-          <t>待审核：干预第14、15次观察的图示读值与正文报告的范围及均值不一致，需核实这两个观察点。</t>
+          <t>Claude补提取（以图为准）：从PDF第6页内嵌原图（1900×2053像素）检测实心菱形（左纵轴，目标儿童回应百分比），按Dyad 3面板刻度（5.395像素/单位）换算。基线9次探测（第1、2、4–9、12次）均为0。图文不一致：干预第14、15次图上为26.1%、38.1%；正文报告均值70.75%、范围33.3–100%，与同伴邀请次数（3次、4次）推算的33.3%、50%相符，图上两点可能绘制有误。按图取值；两种读法下干预期均全部高于基线，Tau-U不受影响。</t>
         </is>
       </c>
     </row>
@@ -20551,10 +20782,24 @@
           <t>Baseline（基线期） vs Intervention（干预期）</t>
         </is>
       </c>
-      <c r="G233" s="33" t="n"/>
-      <c r="H233" s="34" t="n"/>
-      <c r="I233" s="33" t="n"/>
-      <c r="J233" s="34" t="n"/>
+      <c r="G233" s="33" t="inlineStr">
+        <is>
+          <t>0,6,6</t>
+        </is>
+      </c>
+      <c r="H233" s="34">
+        <f>IF(LEN(G233)=0,"",IF(ISNUMBER(SEARCH(",",G233)),LEN(SUBSTITUTE(G233,",","xx"))-LEN(G233)+1,1))</f>
+        <v/>
+      </c>
+      <c r="I233" s="33" t="inlineStr">
+        <is>
+          <t>33,40,66,86,93,100,100,100</t>
+        </is>
+      </c>
+      <c r="J233" s="34">
+        <f>IF(LEN(I233)=0,"",IF(ISNUMBER(SEARCH(",",I233)),LEN(SUBSTITUTE(I233,",","xx"))-LEN(I233)+1,1))</f>
+        <v/>
+      </c>
       <c r="K233" s="13" t="inlineStr">
         <is>
           <t>%</t>
@@ -20565,9 +20810,16 @@
           <t>升高改善</t>
         </is>
       </c>
-      <c r="M233" s="38" t="n"/>
-      <c r="N233" s="38" t="n"/>
-      <c r="O233" s="16" t="n"/>
+      <c r="M233" s="38" t="n">
+        <v>0.816496580927726</v>
+      </c>
+      <c r="N233" s="38" t="n">
+        <v>0.2206713619198469</v>
+      </c>
+      <c r="O233" s="16">
+        <f>IF(AND(N233&lt;0.05,OR(AND(L233="升高改善",M233&gt;0),AND(L233="降低改善",M233&lt;0))),"校正","不校正")</f>
+        <v/>
+      </c>
       <c r="P233" s="13" t="inlineStr">
         <is>
           <t>Figure 1，PDF第27页／印刷页645；Murat 上方面板；纵轴“Correct response percentage”，实心菱形；Baseline与Intervention使用连线，Maintenance为右侧未连接的3个菱形（正文说明干预后1、2、4周，PDF第28页／646）。</t>
@@ -20575,17 +20827,17 @@
       </c>
       <c r="Q233" s="13" t="inlineStr">
         <is>
-          <t>GPT</t>
+          <t>Claude</t>
         </is>
       </c>
       <c r="R233" s="35" t="inlineStr">
         <is>
-          <t>待审核</t>
+          <t>Claude补提取</t>
         </is>
       </c>
       <c r="S233" s="13" t="inlineStr">
         <is>
-          <t>待审核：基线三个图示点的均值与正文报告不一致，尚不能确定哪个点或文字记录有误，需核实整个基线。</t>
+          <t>Claude补提取（以图为准）：Figure 1为PDF矢量图，直接读取Murat面板数据折线顶点的PDF坐标。注意纵轴从−10开始（刻度−10,0,10,…,100），按0与100刻度线换算。基线0,6,6与土耳其文正文（第1次0%，第2、3次6%）一致；英文摘要段写基线均值2%（范围0–6%），按图均值为4%，属图文不一致，按图取值。干预8点均值77.25%，与正文77%（33–100%）一致。原先的“均值不一致”可能是把−10刻度当作0读数所致。</t>
         </is>
       </c>
     </row>
@@ -20620,10 +20872,24 @@
           <t>Baseline（基线期） vs Maintenance（维持期）</t>
         </is>
       </c>
-      <c r="G234" s="22" t="n"/>
-      <c r="H234" s="23" t="n"/>
-      <c r="I234" s="22" t="n"/>
-      <c r="J234" s="23" t="n"/>
+      <c r="G234" s="22" t="inlineStr">
+        <is>
+          <t>0,6,6</t>
+        </is>
+      </c>
+      <c r="H234" s="23">
+        <f>IF(LEN(G234)=0,"",IF(ISNUMBER(SEARCH(",",G234)),LEN(SUBSTITUTE(G234,",","xx"))-LEN(G234)+1,1))</f>
+        <v/>
+      </c>
+      <c r="I234" s="22" t="inlineStr">
+        <is>
+          <t>100,100,100</t>
+        </is>
+      </c>
+      <c r="J234" s="23">
+        <f>IF(LEN(I234)=0,"",IF(ISNUMBER(SEARCH(",",I234)),LEN(SUBSTITUTE(I234,",","xx"))-LEN(I234)+1,1))</f>
+        <v/>
+      </c>
       <c r="K234" s="18" t="inlineStr">
         <is>
           <t>%</t>
@@ -20634,9 +20900,16 @@
           <t>升高改善</t>
         </is>
       </c>
-      <c r="M234" s="39" t="n"/>
-      <c r="N234" s="39" t="n"/>
-      <c r="O234" s="21" t="n"/>
+      <c r="M234" s="39" t="n">
+        <v>0.816496580927726</v>
+      </c>
+      <c r="N234" s="39" t="n">
+        <v>0.2206713619198469</v>
+      </c>
+      <c r="O234" s="21">
+        <f>IF(AND(N234&lt;0.05,OR(AND(L234="升高改善",M234&gt;0),AND(L234="降低改善",M234&lt;0))),"校正","不校正")</f>
+        <v/>
+      </c>
       <c r="P234" s="18" t="inlineStr">
         <is>
           <t>Figure 1，PDF第27页／印刷页645；Murat 上方面板；纵轴“Correct response percentage”，实心菱形；Baseline与Intervention使用连线，Maintenance为右侧未连接的3个菱形（正文说明干预后1、2、4周，PDF第28页／646）。</t>
@@ -20644,17 +20917,17 @@
       </c>
       <c r="Q234" s="18" t="inlineStr">
         <is>
-          <t>GPT</t>
+          <t>Claude</t>
         </is>
       </c>
       <c r="R234" s="24" t="inlineStr">
         <is>
-          <t>待审核</t>
+          <t>Claude补提取</t>
         </is>
       </c>
       <c r="S234" s="18" t="inlineStr">
         <is>
-          <t>待审核：基线三个图示点的均值与正文报告不一致，尚不能确定哪个点或文字记录有误，需核实整个基线。</t>
+          <t>Claude补提取（以图为准）：Figure 1为PDF矢量图，直接读取Murat面板数据折线顶点的PDF坐标。注意纵轴从−10开始（刻度−10,0,10,…,100），按0与100刻度线换算。基线同D0232。维持3次均为100%，与正文一致。</t>
         </is>
       </c>
     </row>
@@ -25534,10 +25807,24 @@
           <t>Post-Training（培训后阶段） vs Maintenance（维持期）</t>
         </is>
       </c>
-      <c r="G291" s="22" t="n"/>
-      <c r="H291" s="23" t="n"/>
-      <c r="I291" s="22" t="n"/>
-      <c r="J291" s="23" t="n"/>
+      <c r="G291" s="22" t="inlineStr">
+        <is>
+          <t>20,25,20,30,30,30,30,30,50,50,30,50,50,50</t>
+        </is>
+      </c>
+      <c r="H291" s="23">
+        <f>IF(LEN(G291)=0,"",IF(ISNUMBER(SEARCH(",",G291)),LEN(SUBSTITUTE(G291,",","xx"))-LEN(G291)+1,1))</f>
+        <v/>
+      </c>
+      <c r="I291" s="22" t="inlineStr">
+        <is>
+          <t>90,75,80,80,80</t>
+        </is>
+      </c>
+      <c r="J291" s="23">
+        <f>IF(LEN(I291)=0,"",IF(ISNUMBER(SEARCH(",",I291)),LEN(SUBSTITUTE(I291,",","xx"))-LEN(I291)+1,1))</f>
+        <v/>
+      </c>
       <c r="K291" s="18" t="inlineStr">
         <is>
           <t>%</t>
@@ -25550,7 +25837,10 @@
       </c>
       <c r="M291" s="39" t="n"/>
       <c r="N291" s="39" t="n"/>
-      <c r="O291" s="21" t="n"/>
+      <c r="O291" s="21">
+        <f>IF(AND(N291&lt;0.05,OR(AND(L291="升高改善",M291&gt;0),AND(L291="降低改善",M291&lt;0))),"校正","不校正")</f>
+        <v/>
+      </c>
       <c r="P291" s="18" t="inlineStr">
         <is>
           <t>Figure 2；PDF第18页，印刷页18 of 28；从上到下第3个Child 3面板；纵轴Percentage of Unprompted Correct Child Responses；目标情境为实心菱形，按Post-Training与Maintenance阶段竖线定位。</t>
@@ -25558,17 +25848,17 @@
       </c>
       <c r="Q291" s="18" t="inlineStr">
         <is>
-          <t>GPT</t>
+          <t>Claude</t>
         </is>
       </c>
       <c r="R291" s="24" t="inlineStr">
         <is>
-          <t>待审核</t>
+          <t>Claude补提取</t>
         </is>
       </c>
       <c r="S291" s="18" t="inlineStr">
         <is>
-          <t>待审核：维持阶段五个图示点与正文报告的数值范围冲突，无法定位具体错误点，需核实完整维持序列。</t>
+          <t>Claude补提取（以图为准）：从PDF第18页内嵌原图（1456×2825像素）检测Child 3面板实心菱形，按该面板0与100位置换算。前段与D0289相同（Post-Training阶段，按一览表约定作为对照段）。维持期为第37、40、42、45、48次5点：90,75,80,80,80，均值81%，与正文M=81%一致；正文范围写60–100%，图上为75–90%，属图文不一致，按图取值。第34、39次圆点为泛化探测，未计入。前段为Post-Training，与同组D0285–D0289保持一致，暂不检验基线趋势（τ、p留空）；是否对030-A的前段做趋势检验待作者确定（如做，此行τ=0.767、p=0.001，需校正）。</t>
         </is>
       </c>
     </row>
@@ -28255,7 +28545,11 @@
           <t>已提取</t>
         </is>
       </c>
-      <c r="S322" s="8" t="n"/>
+      <c r="S322" s="8" t="inlineStr">
+        <is>
+          <t>【Claude复核提示】基线第4次实心圆按矢量形状判断应为3（GPT记为2）：该处圆在上、方块在下，方块为回应=2。按3计，两次基线的发起均值为0.82，按2计为0.73，正文报告0.9（0–3）。建议核对，数值未改。</t>
+        </is>
+      </c>
     </row>
     <row r="323" ht="60" customHeight="1">
       <c r="A323" s="7" t="inlineStr">
@@ -28427,7 +28721,11 @@
           <t>已提取</t>
         </is>
       </c>
-      <c r="S324" s="8" t="n"/>
+      <c r="S324" s="8" t="inlineStr">
+        <is>
+          <t>【Claude复核提示】基线第4次发起值同D0321，可能应为3而非2，建议核对，数值未改。</t>
+        </is>
+      </c>
     </row>
     <row r="325" ht="60" customHeight="1">
       <c r="A325" s="7" t="inlineStr">
@@ -28721,10 +29019,24 @@
           <t>Baseline (first phase)（第一次基线期） vs Intervention (first phase)（第一次干预期）</t>
         </is>
       </c>
-      <c r="G328" s="22" t="n"/>
-      <c r="H328" s="23" t="n"/>
-      <c r="I328" s="22" t="n"/>
-      <c r="J328" s="23" t="n"/>
+      <c r="G328" s="22" t="inlineStr">
+        <is>
+          <t>0,0,0,2,0,0,0,0</t>
+        </is>
+      </c>
+      <c r="H328" s="23">
+        <f>IF(LEN(G328)=0,"",IF(ISNUMBER(SEARCH(",",G328)),LEN(SUBSTITUTE(G328,",","xx"))-LEN(G328)+1,1))</f>
+        <v/>
+      </c>
+      <c r="I328" s="22" t="inlineStr">
+        <is>
+          <t>44,24,16,5,22,26,15</t>
+        </is>
+      </c>
+      <c r="J328" s="23">
+        <f>IF(LEN(I328)=0,"",IF(ISNUMBER(SEARCH(",",I328)),LEN(SUBSTITUTE(I328,",","xx"))-LEN(I328)+1,1))</f>
+        <v/>
+      </c>
       <c r="K328" s="8" t="inlineStr">
         <is>
           <t>次/10分钟</t>
@@ -28735,9 +29047,16 @@
           <t>升高改善</t>
         </is>
       </c>
-      <c r="M328" s="39" t="n"/>
-      <c r="N328" s="39" t="n"/>
-      <c r="O328" s="21" t="n"/>
+      <c r="M328" s="39" t="n">
+        <v>-0.07142857142857142</v>
+      </c>
+      <c r="N328" s="39" t="n">
+        <v>0.8272593465627113</v>
+      </c>
+      <c r="O328" s="21">
+        <f>IF(AND(N328&lt;0.05,OR(AND(L328="升高改善",M328&gt;0),AND(L328="降低改善",M328&lt;0))),"校正","不校正")</f>
+        <v/>
+      </c>
       <c r="P328" s="8" t="inlineStr">
         <is>
           <t>Figure 1；PDF第9页，印刷页9；从上至下第2个Emmett面板；实心方块；图例Responses；空心标记代表与novel peer的泛化观测；按两组Baseline/Intervention竖线区分第一/第二次阶段。</t>
@@ -28745,17 +29064,17 @@
       </c>
       <c r="Q328" s="8" t="inlineStr">
         <is>
-          <t>GPT</t>
+          <t>Claude</t>
         </is>
       </c>
       <c r="R328" s="24" t="inlineStr">
         <is>
-          <t>待审核</t>
+          <t>Claude补提取</t>
         </is>
       </c>
       <c r="S328" s="8" t="inlineStr">
         <is>
-          <t>待审核：基线第4次社交回应的图示读值超出正文报告范围，需核实该点后确认所用基线。</t>
+          <t>Claude补提取（以图为准）：从PDF第9页内嵌原图（1070×1290像素）逐像素检测Emmett面板的实心方块（社交回应），纵轴按PDF中刻度标签位置换算（5.75像素/单位）。第一次基线8点（第1–4、6–9次；第5次为空心泛化探测，未计入）。第4次两个符号重叠：上方为圆（发起=3），下方为方块（回应=2），按形状区分。由此回应基线范围0–2，与正文“0.4次（0–2）”一致，原先所说的“超出正文范围”是把两个符号认反了。第一次干预期7点（第14、17次为泛化探测，未计入），第13次方块与圆重叠，按方块下缘推算为5；与第二次干预期合计14点均值18.0，与正文“18次（5–44）”一致。</t>
         </is>
       </c>
     </row>
@@ -28876,10 +29195,24 @@
           <t>Baseline (first phase)（第一次基线期） vs 6 week follow-up（6周追踪）</t>
         </is>
       </c>
-      <c r="G330" s="22" t="n"/>
-      <c r="H330" s="23" t="n"/>
-      <c r="I330" s="22" t="n"/>
-      <c r="J330" s="23" t="n"/>
+      <c r="G330" s="22" t="inlineStr">
+        <is>
+          <t>0,0,0,2,0,0,0,0</t>
+        </is>
+      </c>
+      <c r="H330" s="23">
+        <f>IF(LEN(G330)=0,"",IF(ISNUMBER(SEARCH(",",G330)),LEN(SUBSTITUTE(G330,",","xx"))-LEN(G330)+1,1))</f>
+        <v/>
+      </c>
+      <c r="I330" s="22" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="J330" s="23">
+        <f>IF(LEN(I330)=0,"",IF(ISNUMBER(SEARCH(",",I330)),LEN(SUBSTITUTE(I330,",","xx"))-LEN(I330)+1,1))</f>
+        <v/>
+      </c>
       <c r="K330" s="8" t="inlineStr">
         <is>
           <t>次/10分钟</t>
@@ -28890,9 +29223,16 @@
           <t>升高改善</t>
         </is>
       </c>
-      <c r="M330" s="39" t="n"/>
-      <c r="N330" s="39" t="n"/>
-      <c r="O330" s="21" t="n"/>
+      <c r="M330" s="39" t="n">
+        <v>-0.07142857142857142</v>
+      </c>
+      <c r="N330" s="39" t="n">
+        <v>0.8272593465627113</v>
+      </c>
+      <c r="O330" s="21">
+        <f>IF(AND(N330&lt;0.05,OR(AND(L330="升高改善",M330&gt;0),AND(L330="降低改善",M330&lt;0))),"校正","不校正")</f>
+        <v/>
+      </c>
       <c r="P330" s="8" t="inlineStr">
         <is>
           <t>Figure 1；PDF第9页，印刷页9；从上至下第2个Emmett面板；实心方块；图例Responses；空心标记代表与novel peer的泛化观测；右侧6 week follow-up区域。</t>
@@ -28900,17 +29240,17 @@
       </c>
       <c r="Q330" s="8" t="inlineStr">
         <is>
-          <t>GPT</t>
+          <t>Claude</t>
         </is>
       </c>
       <c r="R330" s="24" t="inlineStr">
         <is>
-          <t>待审核</t>
+          <t>Claude补提取</t>
         </is>
       </c>
       <c r="S330" s="8" t="inlineStr">
         <is>
-          <t>待审核：基线第4次社交回应的图示读值超出正文报告范围，需核实该点后确认所用基线。</t>
+          <t>Claude补提取（以图为准）：从PDF第9页内嵌原图（1070×1290像素）逐像素检测Emmett面板的实心方块（社交回应），纵轴按PDF中刻度标签位置换算（5.75像素/单位）。基线同D0327。6周追踪的常规会话最右侧实心方块与实心圆重叠，按方块上缘推算为10（圆为9）；与新同伴的泛化追踪为18，两者均值14、范围10–18，与正文一致。追踪只有1点（&lt;3点规则待定）。</t>
         </is>
       </c>
     </row>
@@ -31199,18 +31539,32 @@
       </c>
       <c r="E357" s="13" t="inlineStr">
         <is>
-          <t>待审核</t>
+          <t>干预</t>
         </is>
       </c>
       <c r="F357" s="29" t="inlineStr">
         <is>
-          <t>待审核：Baseline（基线期） / VP Intervention（视频提示干预） / Maintenance（维持期）（原图阶段词；归属未定）</t>
-        </is>
-      </c>
-      <c r="G357" s="33" t="n"/>
-      <c r="H357" s="34" t="n"/>
-      <c r="I357" s="33" t="n"/>
-      <c r="J357" s="34" t="n"/>
+          <t>Baseline（基线期） vs VP Intervention（视频提示干预）</t>
+        </is>
+      </c>
+      <c r="G357" s="33" t="inlineStr">
+        <is>
+          <t>33,25,25,10,30,30</t>
+        </is>
+      </c>
+      <c r="H357" s="34">
+        <f>IF(LEN(G357)=0,"",IF(ISNUMBER(SEARCH(",",G357)),LEN(SUBSTITUTE(G357,",","xx"))-LEN(G357)+1,1))</f>
+        <v/>
+      </c>
+      <c r="I357" s="33" t="inlineStr">
+        <is>
+          <t>60,70,90,80,75,100</t>
+        </is>
+      </c>
+      <c r="J357" s="34">
+        <f>IF(LEN(I357)=0,"",IF(ISNUMBER(SEARCH(",",I357)),LEN(SUBSTITUTE(I357,",","xx"))-LEN(I357)+1,1))</f>
+        <v/>
+      </c>
       <c r="K357" s="13" t="inlineStr">
         <is>
           <t>%</t>
@@ -31221,9 +31575,16 @@
           <t>升高改善</t>
         </is>
       </c>
-      <c r="M357" s="38" t="n"/>
-      <c r="N357" s="38" t="n"/>
-      <c r="O357" s="16" t="n"/>
+      <c r="M357" s="38" t="n">
+        <v>-0.07161148740394328</v>
+      </c>
+      <c r="N357" s="38" t="n">
+        <v>0.8454939839779005</v>
+      </c>
+      <c r="O357" s="16">
+        <f>IF(AND(N357&lt;0.05,OR(AND(L357="升高改善",M357&gt;0),AND(L357="降低改善",M357&lt;0))),"校正","不校正")</f>
+        <v/>
+      </c>
       <c r="P357" s="13" t="inlineStr">
         <is>
           <t>Fig. 1；PDF第9页，所查看图页未标印刷页码；从上至下第3个Mallory Skill 1面板；实心圆为Baseline、VP Intervention和Maintenance数据；空心方块为generalization mean data，非逐次测量；纵轴Percent of Correct Responses。</t>
@@ -31231,17 +31592,17 @@
       </c>
       <c r="Q357" s="13" t="inlineStr">
         <is>
-          <t>GPT</t>
+          <t>Claude</t>
         </is>
       </c>
       <c r="R357" s="35" t="inlineStr">
         <is>
-          <t>待审核</t>
+          <t>Claude补提取</t>
         </is>
       </c>
       <c r="S357" s="13" t="inlineStr">
         <is>
-          <t>待审核：图中阶段线分出6个干预点和5个维持点，正文对应为9个和2个，干预与维持边界尚未确定。</t>
+          <t>Claude补提取（以图为准）：Fig. 1为PDF矢量图，读取实心圆的PDF坐标，按各面板纵轴刻度线（0与100）换算后取整；阶段按图上的实线（基线→视频提示）和虚线（视频提示→维持）划分。Mallory技能1：基线6点均值25.5%，与正文25.5%（10–33%）一致。图文不一致：图上虚线把干预分为6点、维持5点（80,90,100,95,100）；正文干预均值82.78%正是图上干预6点加维持前3点共9点的均值，维持“95–100%”对应最后2点，说明正文的阶段划分与图不同。按图取干预6点。原比较类型“待审核”改为干预比较；如需维持效应，可另加一行：基线 vs 维持80,90,100,95,100。</t>
         </is>
       </c>
     </row>
@@ -31268,18 +31629,32 @@
       </c>
       <c r="E358" s="18" t="inlineStr">
         <is>
-          <t>待审核</t>
+          <t>干预</t>
         </is>
       </c>
       <c r="F358" s="30" t="inlineStr">
         <is>
-          <t>待审核：Baseline（基线期） / VP Intervention（视频提示干预） / Maintenance（维持期）（原图阶段词；归属未定）</t>
-        </is>
-      </c>
-      <c r="G358" s="22" t="n"/>
-      <c r="H358" s="23" t="n"/>
-      <c r="I358" s="22" t="n"/>
-      <c r="J358" s="23" t="n"/>
+          <t>Baseline（基线期） vs VP Intervention（视频提示干预）</t>
+        </is>
+      </c>
+      <c r="G358" s="22" t="inlineStr">
+        <is>
+          <t>40,20,20,20,10,0,40,40</t>
+        </is>
+      </c>
+      <c r="H358" s="23">
+        <f>IF(LEN(G358)=0,"",IF(ISNUMBER(SEARCH(",",G358)),LEN(SUBSTITUTE(G358,",","xx"))-LEN(G358)+1,1))</f>
+        <v/>
+      </c>
+      <c r="I358" s="22" t="inlineStr">
+        <is>
+          <t>60,60,100,100</t>
+        </is>
+      </c>
+      <c r="J358" s="23">
+        <f>IF(LEN(I358)=0,"",IF(ISNUMBER(SEARCH(",",I358)),LEN(SUBSTITUTE(I358,",","xx"))-LEN(I358)+1,1))</f>
+        <v/>
+      </c>
       <c r="K358" s="18" t="inlineStr">
         <is>
           <t>%</t>
@@ -31290,9 +31665,16 @@
           <t>升高改善</t>
         </is>
       </c>
-      <c r="M358" s="39" t="n"/>
-      <c r="N358" s="39" t="n"/>
-      <c r="O358" s="21" t="n"/>
+      <c r="M358" s="39" t="n">
+        <v>-0.08058229640253801</v>
+      </c>
+      <c r="N358" s="39" t="n">
+        <v>0.7928489826282048</v>
+      </c>
+      <c r="O358" s="21">
+        <f>IF(AND(N358&lt;0.05,OR(AND(L358="升高改善",M358&gt;0),AND(L358="降低改善",M358&lt;0))),"校正","不校正")</f>
+        <v/>
+      </c>
       <c r="P358" s="18" t="inlineStr">
         <is>
           <t>Fig. 1；PDF第9页，所查看图页未标印刷页码；从上至下第4个Mallory Skill 2面板；实心圆为Baseline、VP Intervention和Maintenance数据；空心方块为generalization mean data，非逐次测量；纵轴Percent of Correct Responses。</t>
@@ -31300,17 +31682,17 @@
       </c>
       <c r="Q358" s="18" t="inlineStr">
         <is>
-          <t>GPT</t>
+          <t>Claude</t>
         </is>
       </c>
       <c r="R358" s="24" t="inlineStr">
         <is>
-          <t>待审核</t>
+          <t>Claude补提取</t>
         </is>
       </c>
       <c r="S358" s="18" t="inlineStr">
         <is>
-          <t>待审核：图中干预与维持点数为4个和2个，正文对应为5个和1个，且基线均值与正文不符、横轴未标会话号。</t>
+          <t>Claude补提取（以图为准）：Fig. 1为PDF矢量图，读取实心圆的PDF坐标，按各面板纵轴刻度线（0与100）换算后取整；阶段按图上的实线（基线→视频提示）和虚线（视频提示→维持）划分。Mallory技能2：基线8点（空心方块为泛化探测，未计入），均值23.75%，正文21.22%（0–40%）。干预4点均值80%，正文84%（60–100%），正文均值与图上干预4点加维持第1点共5点的均值一致；横轴未标会话号，不影响Tau-U。图文不一致，按图取值。原比较类型“待审核”改为干预比较；维持期图上为100,100（另1个空心方块60%为泛化探测）。</t>
         </is>
       </c>
     </row>
@@ -31337,18 +31719,32 @@
       </c>
       <c r="E359" s="18" t="inlineStr">
         <is>
-          <t>待审核</t>
+          <t>干预</t>
         </is>
       </c>
       <c r="F359" s="30" t="inlineStr">
         <is>
-          <t>待审核：Baseline（基线期） / VP Intervention（视频提示干预） / Maintenance（维持期）（原图阶段词；归属未定）</t>
-        </is>
-      </c>
-      <c r="G359" s="22" t="n"/>
-      <c r="H359" s="23" t="n"/>
-      <c r="I359" s="22" t="n"/>
-      <c r="J359" s="23" t="n"/>
+          <t>Baseline（基线期） vs VP Intervention（视频提示干预）</t>
+        </is>
+      </c>
+      <c r="G359" s="22" t="inlineStr">
+        <is>
+          <t>0,0,0,0,0,0,0,0,0</t>
+        </is>
+      </c>
+      <c r="H359" s="23">
+        <f>IF(LEN(G359)=0,"",IF(ISNUMBER(SEARCH(",",G359)),LEN(SUBSTITUTE(G359,",","xx"))-LEN(G359)+1,1))</f>
+        <v/>
+      </c>
+      <c r="I359" s="22" t="inlineStr">
+        <is>
+          <t>10,80,80,100,100</t>
+        </is>
+      </c>
+      <c r="J359" s="23">
+        <f>IF(LEN(I359)=0,"",IF(ISNUMBER(SEARCH(",",I359)),LEN(SUBSTITUTE(I359,",","xx"))-LEN(I359)+1,1))</f>
+        <v/>
+      </c>
       <c r="K359" s="18" t="inlineStr">
         <is>
           <t>%</t>
@@ -31359,9 +31755,16 @@
           <t>升高改善</t>
         </is>
       </c>
-      <c r="M359" s="39" t="n"/>
-      <c r="N359" s="39" t="n"/>
-      <c r="O359" s="21" t="n"/>
+      <c r="M359" s="39" t="n">
+        <v>0</v>
+      </c>
+      <c r="N359" s="39" t="n">
+        <v>1</v>
+      </c>
+      <c r="O359" s="21">
+        <f>IF(AND(N359&lt;0.05,OR(AND(L359="升高改善",M359&gt;0),AND(L359="降低改善",M359&lt;0))),"校正","不校正")</f>
+        <v/>
+      </c>
       <c r="P359" s="18" t="inlineStr">
         <is>
           <t>Fig. 1；PDF第9页，所查看图页未标印刷页码；从上至下第5个Mateo Skill 1面板；实心圆为Baseline、VP Intervention和Maintenance数据；空心方块为generalization mean data，非逐次测量；纵轴Percent of Correct Responses。</t>
@@ -31369,17 +31772,17 @@
       </c>
       <c r="Q359" s="18" t="inlineStr">
         <is>
-          <t>GPT</t>
+          <t>Claude</t>
         </is>
       </c>
       <c r="R359" s="24" t="inlineStr">
         <is>
-          <t>待审核</t>
+          <t>Claude补提取</t>
         </is>
       </c>
       <c r="S359" s="18" t="inlineStr">
         <is>
-          <t>待审核：方法称未测维持，图末两点却被结果段描述为追踪数据，阶段归属矛盾，需确认干预与维持边界。</t>
+          <t>Claude补提取（以图为准）：Fig. 1为PDF矢量图，读取实心圆的PDF坐标，按各面板纵轴刻度线（0与100）换算后取整；阶段按图上的实线（基线→视频提示）和虚线（视频提示→维持）划分。Mateo技能1：基线9点均为0；干预5点均值74%，与正文74%（10–100%）一致。图文不一致：正文基线均值1%（范围0–10%），图上基线全为0；正文称未测维持，但图上虚线后有2点（100,90，均值95%，与结果段“维持95%”一致）。按图取值。原比较类型“待审核”改为干预比较；如需维持效应，可另加一行：基线 vs 维持100,90。</t>
         </is>
       </c>
     </row>
@@ -31414,10 +31817,24 @@
           <t>Baseline（基线期） vs VP Intervention（视频提示干预）</t>
         </is>
       </c>
-      <c r="G360" s="22" t="n"/>
-      <c r="H360" s="23" t="n"/>
-      <c r="I360" s="22" t="n"/>
-      <c r="J360" s="23" t="n"/>
+      <c r="G360" s="22" t="inlineStr">
+        <is>
+          <t>12,12,0,0,40,0,0,0,0,0</t>
+        </is>
+      </c>
+      <c r="H360" s="23">
+        <f>IF(LEN(G360)=0,"",IF(ISNUMBER(SEARCH(",",G360)),LEN(SUBSTITUTE(G360,",","xx"))-LEN(G360)+1,1))</f>
+        <v/>
+      </c>
+      <c r="I360" s="22" t="inlineStr">
+        <is>
+          <t>31,60,60,60</t>
+        </is>
+      </c>
+      <c r="J360" s="23">
+        <f>IF(LEN(I360)=0,"",IF(ISNUMBER(SEARCH(",",I360)),LEN(SUBSTITUTE(I360,",","xx"))-LEN(I360)+1,1))</f>
+        <v/>
+      </c>
       <c r="K360" s="18" t="inlineStr">
         <is>
           <t>%</t>
@@ -31428,9 +31845,16 @@
           <t>升高改善</t>
         </is>
       </c>
-      <c r="M360" s="39" t="n"/>
-      <c r="N360" s="39" t="n"/>
-      <c r="O360" s="21" t="n"/>
+      <c r="M360" s="39" t="n">
+        <v>-0.4662524041201569</v>
+      </c>
+      <c r="N360" s="39" t="n">
+        <v>0.09284922807157968</v>
+      </c>
+      <c r="O360" s="21">
+        <f>IF(AND(N360&lt;0.05,OR(AND(L360="升高改善",M360&gt;0),AND(L360="降低改善",M360&lt;0))),"校正","不校正")</f>
+        <v/>
+      </c>
       <c r="P360" s="18" t="inlineStr">
         <is>
           <t>Fig. 1；PDF第9页，所查看图页未标印刷页码；从上至下第6个Mateo Skill 2面板；实心圆为Baseline、VP Intervention和Maintenance数据；空心方块为generalization mean data，非逐次测量；纵轴Percent of Correct Responses。</t>
@@ -31438,17 +31862,17 @@
       </c>
       <c r="Q360" s="18" t="inlineStr">
         <is>
-          <t>GPT</t>
+          <t>Claude</t>
         </is>
       </c>
       <c r="R360" s="24" t="inlineStr">
         <is>
-          <t>待审核</t>
+          <t>Claude补提取</t>
         </is>
       </c>
       <c r="S360" s="18" t="inlineStr">
         <is>
-          <t>待审核：基线图示均值与正文报告不一致，无法定位具体错误点，且横轴未印会话数字，确切会话号需核实。</t>
+          <t>Claude补提取（以图为准）：Fig. 1为PDF矢量图，读取实心圆的PDF坐标，按各面板纵轴刻度线（0与100）换算后取整；阶段按图上的实线（基线→视频提示）和虚线（视频提示→维持）划分。Mateo技能2：基线10点（横轴未标会话号，只按先后取值），均值6.4%；正文基线均值7.9%（0–40%），图文不一致，无法定位，按图取值。干预4点：图上第1点约31%，正文干预均值52.5%（30–60%）对应第1点为30%，差1个百分点，不影响Tau-U。</t>
         </is>
       </c>
     </row>
@@ -32519,10 +32943,24 @@
           <t>Baseline（基线期） vs Maintenance（维持期）</t>
         </is>
       </c>
-      <c r="G373" s="22" t="n"/>
-      <c r="H373" s="23" t="n"/>
-      <c r="I373" s="22" t="n"/>
-      <c r="J373" s="23" t="n"/>
+      <c r="G373" s="22" t="inlineStr">
+        <is>
+          <t>0,0,0,0,0,0</t>
+        </is>
+      </c>
+      <c r="H373" s="23">
+        <f>IF(LEN(G373)=0,"",IF(ISNUMBER(SEARCH(",",G373)),LEN(SUBSTITUTE(G373,",","xx"))-LEN(G373)+1,1))</f>
+        <v/>
+      </c>
+      <c r="I373" s="22" t="inlineStr">
+        <is>
+          <t>12,20,11,6,20</t>
+        </is>
+      </c>
+      <c r="J373" s="23">
+        <f>IF(LEN(I373)=0,"",IF(ISNUMBER(SEARCH(",",I373)),LEN(SUBSTITUTE(I373,",","xx"))-LEN(I373)+1,1))</f>
+        <v/>
+      </c>
       <c r="K373" s="18" t="inlineStr">
         <is>
           <t>次数/观察期</t>
@@ -32533,9 +32971,16 @@
           <t>升高改善</t>
         </is>
       </c>
-      <c r="M373" s="39" t="n"/>
-      <c r="N373" s="39" t="n"/>
-      <c r="O373" s="21" t="n"/>
+      <c r="M373" s="39" t="n">
+        <v>0</v>
+      </c>
+      <c r="N373" s="39" t="n">
+        <v>1</v>
+      </c>
+      <c r="O373" s="21">
+        <f>IF(AND(N373&lt;0.05,OR(AND(L373="升高改善",M373&gt;0),AND(L373="降低改善",M373&lt;0))),"校正","不校正")</f>
+        <v/>
+      </c>
       <c r="P373" s="18" t="inlineStr">
         <is>
           <t>Fig. 1；PDF第9页，所查看图页未标印刷页码；最上方Dyad A（Aaron）面板；右纵轴Frequency of Communication Opportunities and Child Behavior；实心方块（child target communication behavior）；三角形和圆形为教师/沟通机会数据，不属于本行。Aaron目标原文：Request desired or needed item(s) or action(s) from an adult or peer using three or more spoken words。</t>
@@ -32543,17 +32988,17 @@
       </c>
       <c r="Q373" s="18" t="inlineStr">
         <is>
-          <t>GPT</t>
+          <t>Claude</t>
         </is>
       </c>
       <c r="R373" s="24" t="inlineStr">
         <is>
-          <t>待审核</t>
+          <t>Claude补提取</t>
         </is>
       </c>
       <c r="S373" s="18" t="inlineStr">
         <is>
-          <t>待审核：维持阶段五个图示点超出正文报告范围，且相关泛化阶段的图文值疑似对调，需核实阶段和读值。</t>
+          <t>Claude补提取（以图为准）：Fig. 1为PDF矢量图，读取Dyad A实心/空心方块的PDF坐标，按右纵轴（0–25）刻度线换算；干预与维持分界位于第16、17次之间。基线6点与D0371相同。维持期实心方块为第17、21、25、29、33次：12,20,11,6,20（第33次方块上叠了一个无边框白色圆点，渲染后像空心方块，矢量数据显示为实心方块）。图文不一致：正文报告维持范围9–16，图上为6–20；同图Bryan的数据也与正文范围不符，判断为正文问题，按图取值。</t>
         </is>
       </c>
     </row>
@@ -32588,10 +33033,24 @@
           <t>Baseline (Generalization Probes)（基线期的泛化测查） vs Intervention (Generalization Probes)（干预期的泛化测查）</t>
         </is>
       </c>
-      <c r="G374" s="22" t="n"/>
-      <c r="H374" s="23" t="n"/>
-      <c r="I374" s="22" t="n"/>
-      <c r="J374" s="23" t="n"/>
+      <c r="G374" s="22" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="H374" s="23">
+        <f>IF(LEN(G374)=0,"",IF(ISNUMBER(SEARCH(",",G374)),LEN(SUBSTITUTE(G374,",","xx"))-LEN(G374)+1,1))</f>
+        <v/>
+      </c>
+      <c r="I374" s="22" t="inlineStr">
+        <is>
+          <t>13</t>
+        </is>
+      </c>
+      <c r="J374" s="23">
+        <f>IF(LEN(I374)=0,"",IF(ISNUMBER(SEARCH(",",I374)),LEN(SUBSTITUTE(I374,",","xx"))-LEN(I374)+1,1))</f>
+        <v/>
+      </c>
       <c r="K374" s="18" t="inlineStr">
         <is>
           <t>次数/观察期</t>
@@ -32602,9 +33061,16 @@
           <t>升高改善</t>
         </is>
       </c>
-      <c r="M374" s="39" t="n"/>
-      <c r="N374" s="39" t="n"/>
-      <c r="O374" s="21" t="n"/>
+      <c r="M374" s="39" t="n">
+        <v>0</v>
+      </c>
+      <c r="N374" s="39" t="n">
+        <v>1</v>
+      </c>
+      <c r="O374" s="21">
+        <f>IF(AND(N374&lt;0.05,OR(AND(L374="升高改善",M374&gt;0),AND(L374="降低改善",M374&lt;0))),"校正","不校正")</f>
+        <v/>
+      </c>
       <c r="P374" s="18" t="inlineStr">
         <is>
           <t>Fig. 1；PDF第9页，所查看图页未标印刷页码；最上方Dyad A（Aaron）面板；右纵轴Frequency of Communication Opportunities and Child Behavior；空心方块（child behavior generalization probes）；三角形和圆形为教师/沟通机会数据，不属于本行。Aaron目标原文：Request desired or needed item(s) or action(s) from an adult or peer using three or more spoken words。</t>
@@ -32612,17 +33078,17 @@
       </c>
       <c r="Q374" s="18" t="inlineStr">
         <is>
-          <t>GPT</t>
+          <t>Claude</t>
         </is>
       </c>
       <c r="R374" s="24" t="inlineStr">
         <is>
-          <t>待审核</t>
+          <t>Claude补提取</t>
         </is>
       </c>
       <c r="S374" s="18" t="inlineStr">
         <is>
-          <t>待审核：干预期与维持期的泛化图示值和正文所述疑似对调，尚需确认两个探测点的数值及阶段归属。</t>
+          <t>Claude补提取（以图为准）：Fig. 1为PDF矢量图，读取Dyad A实心/空心方块的PDF坐标，按右纵轴（0–25）刻度线换算；干预与维持分界位于第16、17次之间。泛化探测（空心方块）：基线第5次为0，干预期第16次为13。图文不一致：正文写“干预期10、维持期13”，图上干预期为13、维持期为10，两者疑似对调；按图取值。两段均只有1点（&lt;3点规则待定）。</t>
         </is>
       </c>
     </row>
@@ -32657,10 +33123,24 @@
           <t>Baseline (Generalization Probes)（基线期的泛化测查） vs Maintenance (Generalization Probes)（维持期的泛化测查）</t>
         </is>
       </c>
-      <c r="G375" s="22" t="n"/>
-      <c r="H375" s="23" t="n"/>
-      <c r="I375" s="22" t="n"/>
-      <c r="J375" s="23" t="n"/>
+      <c r="G375" s="22" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="H375" s="23">
+        <f>IF(LEN(G375)=0,"",IF(ISNUMBER(SEARCH(",",G375)),LEN(SUBSTITUTE(G375,",","xx"))-LEN(G375)+1,1))</f>
+        <v/>
+      </c>
+      <c r="I375" s="22" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="J375" s="23">
+        <f>IF(LEN(I375)=0,"",IF(ISNUMBER(SEARCH(",",I375)),LEN(SUBSTITUTE(I375,",","xx"))-LEN(I375)+1,1))</f>
+        <v/>
+      </c>
       <c r="K375" s="18" t="inlineStr">
         <is>
           <t>次数/观察期</t>
@@ -32671,9 +33151,16 @@
           <t>升高改善</t>
         </is>
       </c>
-      <c r="M375" s="39" t="n"/>
-      <c r="N375" s="39" t="n"/>
-      <c r="O375" s="21" t="n"/>
+      <c r="M375" s="39" t="n">
+        <v>0</v>
+      </c>
+      <c r="N375" s="39" t="n">
+        <v>1</v>
+      </c>
+      <c r="O375" s="21">
+        <f>IF(AND(N375&lt;0.05,OR(AND(L375="升高改善",M375&gt;0),AND(L375="降低改善",M375&lt;0))),"校正","不校正")</f>
+        <v/>
+      </c>
       <c r="P375" s="18" t="inlineStr">
         <is>
           <t>Fig. 1；PDF第9页，所查看图页未标印刷页码；最上方Dyad A（Aaron）面板；右纵轴Frequency of Communication Opportunities and Child Behavior；空心方块（child behavior generalization probes）；三角形和圆形为教师/沟通机会数据，不属于本行。Aaron目标原文：Request desired or needed item(s) or action(s) from an adult or peer using three or more spoken words。</t>
@@ -32681,17 +33168,17 @@
       </c>
       <c r="Q375" s="18" t="inlineStr">
         <is>
-          <t>GPT</t>
+          <t>Claude</t>
         </is>
       </c>
       <c r="R375" s="24" t="inlineStr">
         <is>
-          <t>待审核</t>
+          <t>Claude补提取</t>
         </is>
       </c>
       <c r="S375" s="18" t="inlineStr">
         <is>
-          <t>待审核：干预期与维持期的泛化图示值和正文所述疑似对调，尚需确认两个探测点的数值及阶段归属。</t>
+          <t>Claude补提取（以图为准）：Fig. 1为PDF矢量图，读取Dyad A实心/空心方块的PDF坐标，按右纵轴（0–25）刻度线换算；干预与维持分界位于第16、17次之间。泛化探测：基线第5次为0，维持期第34次为10。图文不一致：正文写维持期13，图上为10（与干预期数值疑似对调，见D0373）；按图取值。两段均只有1点（&lt;3点规则待定）。</t>
         </is>
       </c>
     </row>
@@ -37628,10 +38115,24 @@
           <t>Baseline（基线期） vs Intervention（干预期）</t>
         </is>
       </c>
-      <c r="G433" s="33" t="n"/>
-      <c r="H433" s="34" t="n"/>
-      <c r="I433" s="33" t="n"/>
-      <c r="J433" s="34" t="n"/>
+      <c r="G433" s="33" t="inlineStr">
+        <is>
+          <t>20,35,30,25,15,40,45,40,40</t>
+        </is>
+      </c>
+      <c r="H433" s="34">
+        <f>IF(LEN(G433)=0,"",IF(ISNUMBER(SEARCH(",",G433)),LEN(SUBSTITUTE(G433,",","xx"))-LEN(G433)+1,1))</f>
+        <v/>
+      </c>
+      <c r="I433" s="33" t="inlineStr">
+        <is>
+          <t>70,80,90,100,90,120,135,150,140,160,175,180,190,175,180,190,220,250</t>
+        </is>
+      </c>
+      <c r="J433" s="34">
+        <f>IF(LEN(I433)=0,"",IF(ISNUMBER(SEARCH(",",I433)),LEN(SUBSTITUTE(I433,",","xx"))-LEN(I433)+1,1))</f>
+        <v/>
+      </c>
       <c r="K433" s="13" t="inlineStr">
         <is>
           <t>秒</t>
@@ -37642,9 +38143,16 @@
           <t>升高改善</t>
         </is>
       </c>
-      <c r="M433" s="38" t="n"/>
-      <c r="N433" s="38" t="n"/>
-      <c r="O433" s="16" t="n"/>
+      <c r="M433" s="38" t="n">
+        <v>0.4351941398892446</v>
+      </c>
+      <c r="N433" s="38" t="n">
+        <v>0.110492024055668</v>
+      </c>
+      <c r="O433" s="16">
+        <f>IF(AND(N433&lt;0.05,OR(AND(L433="升高改善",M433&gt;0),AND(L433="降低改善",M433&lt;0))),"校正","不校正")</f>
+        <v/>
+      </c>
       <c r="P433" s="13" t="inlineStr">
         <is>
           <t>Fig. 1；PDF第14页，印刷页1134；从上至下第1个Fox面板；实心圆连线，纵轴The Duration of Social Interaction (Seconds)；Baseline与Intervention竖虚线两侧。</t>
@@ -37652,17 +38160,17 @@
       </c>
       <c r="Q433" s="13" t="inlineStr">
         <is>
-          <t>GPT</t>
+          <t>Claude</t>
         </is>
       </c>
       <c r="R433" s="35" t="inlineStr">
         <is>
-          <t>待审核</t>
+          <t>Claude补提取</t>
         </is>
       </c>
       <c r="S433" s="13" t="inlineStr">
         <is>
-          <t>待审核：基线社交互动时长的图示最大值超出表1报告范围，图表不一致，需核实最高观察点。</t>
+          <t>Claude补提取（以图为准）：从PDF第14页Fig. 1内嵌原图（1406×1791像素）逐像素检测实心圆，按各面板纵轴刻度标签换算，读数均落在5秒的整倍数上。Fox基线9点均值32.2，与表1一致；图文不一致：基线第7次图上为45秒，超出表1范围15–40。干预18点均值149.7、范围70–250，与表1一致。按图取值。</t>
         </is>
       </c>
     </row>
@@ -37697,10 +38205,24 @@
           <t>Baseline（基线期） vs Maintenance（维持期）</t>
         </is>
       </c>
-      <c r="G434" s="22" t="n"/>
-      <c r="H434" s="23" t="n"/>
-      <c r="I434" s="22" t="n"/>
-      <c r="J434" s="23" t="n"/>
+      <c r="G434" s="22" t="inlineStr">
+        <is>
+          <t>20,35,30,25,15,40,45,40,40</t>
+        </is>
+      </c>
+      <c r="H434" s="23">
+        <f>IF(LEN(G434)=0,"",IF(ISNUMBER(SEARCH(",",G434)),LEN(SUBSTITUTE(G434,",","xx"))-LEN(G434)+1,1))</f>
+        <v/>
+      </c>
+      <c r="I434" s="22" t="inlineStr">
+        <is>
+          <t>170,180,190,190</t>
+        </is>
+      </c>
+      <c r="J434" s="23">
+        <f>IF(LEN(I434)=0,"",IF(ISNUMBER(SEARCH(",",I434)),LEN(SUBSTITUTE(I434,",","xx"))-LEN(I434)+1,1))</f>
+        <v/>
+      </c>
       <c r="K434" s="18" t="inlineStr">
         <is>
           <t>秒</t>
@@ -37711,9 +38233,16 @@
           <t>升高改善</t>
         </is>
       </c>
-      <c r="M434" s="39" t="n"/>
-      <c r="N434" s="39" t="n"/>
-      <c r="O434" s="21" t="n"/>
+      <c r="M434" s="39" t="n">
+        <v>0.4351941398892446</v>
+      </c>
+      <c r="N434" s="39" t="n">
+        <v>0.110492024055668</v>
+      </c>
+      <c r="O434" s="21">
+        <f>IF(AND(N434&lt;0.05,OR(AND(L434="升高改善",M434&gt;0),AND(L434="降低改善",M434&lt;0))),"校正","不校正")</f>
+        <v/>
+      </c>
       <c r="P434" s="18" t="inlineStr">
         <is>
           <t>Fig. 1；PDF第14页，印刷页1134；从上至下第1个Fox面板；实心圆连线，纵轴The Duration of Social Interaction (Seconds)；右侧Maintenance区域。</t>
@@ -37721,17 +38250,17 @@
       </c>
       <c r="Q434" s="18" t="inlineStr">
         <is>
-          <t>GPT</t>
+          <t>Claude</t>
         </is>
       </c>
       <c r="R434" s="24" t="inlineStr">
         <is>
-          <t>待审核</t>
+          <t>Claude补提取</t>
         </is>
       </c>
       <c r="S434" s="18" t="inlineStr">
         <is>
-          <t>待审核：基线社交互动时长的图示最大值超出表1报告范围，图表不一致，需核实最高观察点。</t>
+          <t>Claude补提取（以图为准）：从PDF第14页Fig. 1内嵌原图（1406×1791像素）逐像素检测实心圆，按各面板纵轴刻度标签换算，读数均落在5秒的整倍数上。基线同D0432（第7次45秒超出表1范围）。维持4点均值182.5、范围170–190，与表1一致。</t>
         </is>
       </c>
     </row>
@@ -37766,10 +38295,24 @@
           <t>Baseline（基线期） vs Intervention（干预期）</t>
         </is>
       </c>
-      <c r="G435" s="22" t="n"/>
-      <c r="H435" s="23" t="n"/>
-      <c r="I435" s="22" t="n"/>
-      <c r="J435" s="23" t="n"/>
+      <c r="G435" s="22" t="inlineStr">
+        <is>
+          <t>2,3,3,5,4,3,4,4,4</t>
+        </is>
+      </c>
+      <c r="H435" s="23">
+        <f>IF(LEN(G435)=0,"",IF(ISNUMBER(SEARCH(",",G435)),LEN(SUBSTITUTE(G435,",","xx"))-LEN(G435)+1,1))</f>
+        <v/>
+      </c>
+      <c r="I435" s="22" t="inlineStr">
+        <is>
+          <t>6,6,8,7,8,8,9,9,8,8,9,7,8,9,8,9,10,10</t>
+        </is>
+      </c>
+      <c r="J435" s="23">
+        <f>IF(LEN(I435)=0,"",IF(ISNUMBER(SEARCH(",",I435)),LEN(SUBSTITUTE(I435,",","xx"))-LEN(I435)+1,1))</f>
+        <v/>
+      </c>
       <c r="K435" s="18" t="inlineStr">
         <is>
           <t>次数</t>
@@ -37780,9 +38323,16 @@
           <t>升高改善</t>
         </is>
       </c>
-      <c r="M435" s="39" t="n"/>
-      <c r="N435" s="39" t="n"/>
-      <c r="O435" s="21" t="n"/>
+      <c r="M435" s="39" t="n">
+        <v>0.4811252243246881</v>
+      </c>
+      <c r="N435" s="39" t="n">
+        <v>0.09284922807157968</v>
+      </c>
+      <c r="O435" s="21">
+        <f>IF(AND(N435&lt;0.05,OR(AND(L435="升高改善",M435&gt;0),AND(L435="降低改善",M435&lt;0))),"校正","不校正")</f>
+        <v/>
+      </c>
       <c r="P435" s="18" t="inlineStr">
         <is>
           <t>Fig. 2；PDF第16页，印刷页1136；从上至下第1个Fox面板；黑色实心方块，图例Initiations；Baseline与Intervention竖虚线两侧。</t>
@@ -37790,17 +38340,17 @@
       </c>
       <c r="Q435" s="18" t="inlineStr">
         <is>
-          <t>GPT</t>
+          <t>Claude</t>
         </is>
       </c>
       <c r="R435" s="24" t="inlineStr">
         <is>
-          <t>待审核</t>
+          <t>Claude补提取</t>
         </is>
       </c>
       <c r="S435" s="18" t="inlineStr">
         <is>
-          <t>待审核：基线第4次观察的图示读值与表1范围冲突，正文范围却支持图示，原文内部不一致，需核实该点。</t>
+          <t>Claude补提取（以图为准）：从PDF第16页Fig. 2内嵌原图（1406×1618像素）逐像素检测黑色方块（发起）和浅灰圆点（回应），按纵轴刻度标签换算，读数均为整数；被浅灰圆点覆盖的方块按图上位置读取。Fox基线9点均值3.56，与表1均值3.60一致；图文不一致：基线第4次图上为5，超出表1范围2–4（正文范围支持图示）。干预18点均值8.17、范围6–10，与表1（8.20，6–10）一致。按图取值。</t>
         </is>
       </c>
     </row>
@@ -37835,10 +38385,24 @@
           <t>Baseline（基线期） vs Maintenance（维持期）</t>
         </is>
       </c>
-      <c r="G436" s="22" t="n"/>
-      <c r="H436" s="23" t="n"/>
-      <c r="I436" s="22" t="n"/>
-      <c r="J436" s="23" t="n"/>
+      <c r="G436" s="22" t="inlineStr">
+        <is>
+          <t>2,3,3,5,4,3,4,4,4</t>
+        </is>
+      </c>
+      <c r="H436" s="23">
+        <f>IF(LEN(G436)=0,"",IF(ISNUMBER(SEARCH(",",G436)),LEN(SUBSTITUTE(G436,",","xx"))-LEN(G436)+1,1))</f>
+        <v/>
+      </c>
+      <c r="I436" s="22" t="inlineStr">
+        <is>
+          <t>7,8,7,7</t>
+        </is>
+      </c>
+      <c r="J436" s="23">
+        <f>IF(LEN(I436)=0,"",IF(ISNUMBER(SEARCH(",",I436)),LEN(SUBSTITUTE(I436,",","xx"))-LEN(I436)+1,1))</f>
+        <v/>
+      </c>
       <c r="K436" s="18" t="inlineStr">
         <is>
           <t>次数</t>
@@ -37849,9 +38413,16 @@
           <t>升高改善</t>
         </is>
       </c>
-      <c r="M436" s="39" t="n"/>
-      <c r="N436" s="39" t="n"/>
-      <c r="O436" s="21" t="n"/>
+      <c r="M436" s="39" t="n">
+        <v>0.4811252243246881</v>
+      </c>
+      <c r="N436" s="39" t="n">
+        <v>0.09284922807157968</v>
+      </c>
+      <c r="O436" s="21">
+        <f>IF(AND(N436&lt;0.05,OR(AND(L436="升高改善",M436&gt;0),AND(L436="降低改善",M436&lt;0))),"校正","不校正")</f>
+        <v/>
+      </c>
       <c r="P436" s="18" t="inlineStr">
         <is>
           <t>Fig. 2；PDF第16页，印刷页1136；从上至下第1个Fox面板；黑色实心方块，图例Initiations；右侧Maintenance区域。</t>
@@ -37859,17 +38430,17 @@
       </c>
       <c r="Q436" s="18" t="inlineStr">
         <is>
-          <t>GPT</t>
+          <t>Claude</t>
         </is>
       </c>
       <c r="R436" s="24" t="inlineStr">
         <is>
-          <t>待审核</t>
+          <t>Claude补提取</t>
         </is>
       </c>
       <c r="S436" s="18" t="inlineStr">
         <is>
-          <t>待审核：基线第4次观察的图示读值与表1范围冲突，正文范围却支持图示，原文内部不一致，需核实该点。</t>
+          <t>Claude补提取（以图为准）：从PDF第16页Fig. 2内嵌原图（1406×1618像素）逐像素检测黑色方块（发起）和浅灰圆点（回应），按纵轴刻度标签换算，读数均为整数；被浅灰圆点覆盖的方块按图上位置读取。基线同D0434。维持4点均值7.25、范围7–8，与表1（7.20，7–8）一致。</t>
         </is>
       </c>
     </row>
@@ -38076,10 +38647,24 @@
           <t>Baseline（基线期） vs Intervention（干预期）</t>
         </is>
       </c>
-      <c r="G439" s="22" t="n"/>
-      <c r="H439" s="23" t="n"/>
-      <c r="I439" s="22" t="n"/>
-      <c r="J439" s="23" t="n"/>
+      <c r="G439" s="22" t="inlineStr">
+        <is>
+          <t>20,15,15,25,20,20,15,25,20,25,25,25</t>
+        </is>
+      </c>
+      <c r="H439" s="23">
+        <f>IF(LEN(G439)=0,"",IF(ISNUMBER(SEARCH(",",G439)),LEN(SUBSTITUTE(G439,",","xx"))-LEN(G439)+1,1))</f>
+        <v/>
+      </c>
+      <c r="I439" s="22" t="inlineStr">
+        <is>
+          <t>55,60,65,85,95,110,100,150,120,160,180,175,190,220,250</t>
+        </is>
+      </c>
+      <c r="J439" s="23">
+        <f>IF(LEN(I439)=0,"",IF(ISNUMBER(SEARCH(",",I439)),LEN(SUBSTITUTE(I439,",","xx"))-LEN(I439)+1,1))</f>
+        <v/>
+      </c>
       <c r="K439" s="18" t="inlineStr">
         <is>
           <t>秒</t>
@@ -38090,9 +38675,16 @@
           <t>升高改善</t>
         </is>
       </c>
-      <c r="M439" s="39" t="n"/>
-      <c r="N439" s="39" t="n"/>
-      <c r="O439" s="21" t="n"/>
+      <c r="M439" s="39" t="n">
+        <v>0.4847779606994154</v>
+      </c>
+      <c r="N439" s="39" t="n">
+        <v>0.04634124184080035</v>
+      </c>
+      <c r="O439" s="21">
+        <f>IF(AND(N439&lt;0.05,OR(AND(L439="升高改善",M439&gt;0),AND(L439="降低改善",M439&lt;0))),"校正","不校正")</f>
+        <v/>
+      </c>
       <c r="P439" s="18" t="inlineStr">
         <is>
           <t>Fig. 1；PDF第14页，印刷页1134；从上至下第2个Sam面板；实心圆连线，纵轴The Duration of Social Interaction (Seconds)；Baseline与Intervention竖虚线两侧。</t>
@@ -38100,17 +38692,17 @@
       </c>
       <c r="Q439" s="18" t="inlineStr">
         <is>
-          <t>GPT</t>
+          <t>Claude</t>
         </is>
       </c>
       <c r="R439" s="24" t="inlineStr">
         <is>
-          <t>待审核</t>
+          <t>Claude补提取</t>
         </is>
       </c>
       <c r="S439" s="18" t="inlineStr">
         <is>
-          <t>待审核：基线图示均值及范围与表1不符，干预末段图示值又超出表1上限，无法定位错误来源，需核实两段数据。</t>
+          <t>Claude补提取（以图为准）：从PDF第14页Fig. 1内嵌原图（1406×1791像素）逐像素检测实心圆，按各面板纵轴刻度标签换算，读数均落在5秒的整倍数上。图文不一致：Sam基线12点均值20.8、范围15–25，表1报告28.7（15–40）；干预15点均值134.3、范围55–250，表1报告133.3（55–200）。表1中Sam基线的均值、SD、范围与Fox高度相似，可能有抄录错误。按图取值。</t>
         </is>
       </c>
     </row>
@@ -38145,10 +38737,24 @@
           <t>Baseline（基线期） vs Maintenance（维持期）</t>
         </is>
       </c>
-      <c r="G440" s="22" t="n"/>
-      <c r="H440" s="23" t="n"/>
-      <c r="I440" s="22" t="n"/>
-      <c r="J440" s="23" t="n"/>
+      <c r="G440" s="22" t="inlineStr">
+        <is>
+          <t>20,15,15,25,20,20,15,25,20,25,25,25</t>
+        </is>
+      </c>
+      <c r="H440" s="23">
+        <f>IF(LEN(G440)=0,"",IF(ISNUMBER(SEARCH(",",G440)),LEN(SUBSTITUTE(G440,",","xx"))-LEN(G440)+1,1))</f>
+        <v/>
+      </c>
+      <c r="I440" s="22" t="inlineStr">
+        <is>
+          <t>200,170,180,200</t>
+        </is>
+      </c>
+      <c r="J440" s="23">
+        <f>IF(LEN(I440)=0,"",IF(ISNUMBER(SEARCH(",",I440)),LEN(SUBSTITUTE(I440,",","xx"))-LEN(I440)+1,1))</f>
+        <v/>
+      </c>
       <c r="K440" s="18" t="inlineStr">
         <is>
           <t>秒</t>
@@ -38159,9 +38765,16 @@
           <t>升高改善</t>
         </is>
       </c>
-      <c r="M440" s="39" t="n"/>
-      <c r="N440" s="39" t="n"/>
-      <c r="O440" s="21" t="n"/>
+      <c r="M440" s="39" t="n">
+        <v>0.4847779606994154</v>
+      </c>
+      <c r="N440" s="39" t="n">
+        <v>0.04634124184080035</v>
+      </c>
+      <c r="O440" s="21">
+        <f>IF(AND(N440&lt;0.05,OR(AND(L440="升高改善",M440&gt;0),AND(L440="降低改善",M440&lt;0))),"校正","不校正")</f>
+        <v/>
+      </c>
       <c r="P440" s="18" t="inlineStr">
         <is>
           <t>Fig. 1；PDF第14页，印刷页1134；从上至下第2个Sam面板；实心圆连线，纵轴The Duration of Social Interaction (Seconds)；右侧Maintenance区域。</t>
@@ -38169,17 +38782,17 @@
       </c>
       <c r="Q440" s="18" t="inlineStr">
         <is>
-          <t>GPT</t>
+          <t>Claude</t>
         </is>
       </c>
       <c r="R440" s="24" t="inlineStr">
         <is>
-          <t>待审核</t>
+          <t>Claude补提取</t>
         </is>
       </c>
       <c r="S440" s="18" t="inlineStr">
         <is>
-          <t>待审核：基线及维持阶段的图示均值、范围均与表1报告不一致，无法定位具体错误点，需核实两个阶段。</t>
+          <t>Claude补提取（以图为准）：从PDF第14页Fig. 1内嵌原图（1406×1791像素）逐像素检测实心圆，按各面板纵轴刻度标签换算，读数均落在5秒的整倍数上。基线同D0438。图文不一致：维持4点均值187.5、范围170–200，表1报告170（160–180）。按图取值。</t>
         </is>
       </c>
     </row>
@@ -38902,10 +39515,24 @@
           <t>Baseline（基线期） vs Intervention（干预期）</t>
         </is>
       </c>
-      <c r="G449" s="22" t="n"/>
-      <c r="H449" s="23" t="n"/>
-      <c r="I449" s="22" t="n"/>
-      <c r="J449" s="23" t="n"/>
+      <c r="G449" s="22" t="inlineStr">
+        <is>
+          <t>1,2,2,3,2,3,3,2,4,3,4,3,2,3,3,3,3</t>
+        </is>
+      </c>
+      <c r="H449" s="23">
+        <f>IF(LEN(G449)=0,"",IF(ISNUMBER(SEARCH(",",G449)),LEN(SUBSTITUTE(G449,",","xx"))-LEN(G449)+1,1))</f>
+        <v/>
+      </c>
+      <c r="I449" s="22" t="inlineStr">
+        <is>
+          <t>5,6,5,6,8,8,7,8,8,9</t>
+        </is>
+      </c>
+      <c r="J449" s="23">
+        <f>IF(LEN(I449)=0,"",IF(ISNUMBER(SEARCH(",",I449)),LEN(SUBSTITUTE(I449,",","xx"))-LEN(I449)+1,1))</f>
+        <v/>
+      </c>
       <c r="K449" s="18" t="inlineStr">
         <is>
           <t>次数</t>
@@ -38916,9 +39543,16 @@
           <t>升高改善</t>
         </is>
       </c>
-      <c r="M449" s="39" t="n"/>
-      <c r="N449" s="39" t="n"/>
-      <c r="O449" s="21" t="n"/>
+      <c r="M449" s="39" t="n">
+        <v>0.4090233075190866</v>
+      </c>
+      <c r="N449" s="39" t="n">
+        <v>0.03991058571027136</v>
+      </c>
+      <c r="O449" s="21">
+        <f>IF(AND(N449&lt;0.05,OR(AND(L449="升高改善",M449&gt;0),AND(L449="降低改善",M449&lt;0))),"校正","不校正")</f>
+        <v/>
+      </c>
       <c r="P449" s="18" t="inlineStr">
         <is>
           <t>Fig. 2；PDF第16页，印刷页1136；从上至下第3个Nia面板；浅灰圆点及浅灰连线，图例Responses；Baseline与Intervention竖虚线两侧。</t>
@@ -38926,17 +39560,17 @@
       </c>
       <c r="Q449" s="18" t="inlineStr">
         <is>
-          <t>GPT</t>
+          <t>Claude</t>
         </is>
       </c>
       <c r="R449" s="24" t="inlineStr">
         <is>
-          <t>待审核</t>
+          <t>Claude补提取</t>
         </is>
       </c>
       <c r="S449" s="18" t="inlineStr">
         <is>
-          <t>待审核：干预图可见10个观察点，其均值与表1报告不符，尚不能判断具体哪些点或表值有误。</t>
+          <t>Claude补提取（以图为准）：从PDF第16页Fig. 2内嵌原图（1406×1618像素）逐像素检测黑色方块（发起）和浅灰圆点（回应），按纵轴刻度标签换算，读数均为整数；被浅灰圆点覆盖的方块按图上位置读取。基线17点与D0449相同。图文不一致：干预10点均值7.0，表1报告7.70（范围5–9与图一致），无法定位具体哪个点，按图取值。</t>
         </is>
       </c>
     </row>
@@ -39057,10 +39691,24 @@
           <t>Baseline（基线期） vs Intervention（干预期）</t>
         </is>
       </c>
-      <c r="G451" s="33" t="n"/>
-      <c r="H451" s="34" t="n"/>
-      <c r="I451" s="33" t="n"/>
-      <c r="J451" s="34" t="n"/>
+      <c r="G451" s="33" t="inlineStr">
+        <is>
+          <t>0,0,0,0</t>
+        </is>
+      </c>
+      <c r="H451" s="34">
+        <f>IF(LEN(G451)=0,"",IF(ISNUMBER(SEARCH(",",G451)),LEN(SUBSTITUTE(G451,",","xx"))-LEN(G451)+1,1))</f>
+        <v/>
+      </c>
+      <c r="I451" s="33" t="inlineStr">
+        <is>
+          <t>100,88,100,100,100,100,100,80,90,100,87,53,65,60,75,100,55,100,100,73,93,80,80,100,92,100,85,100,70,95</t>
+        </is>
+      </c>
+      <c r="J451" s="34">
+        <f>IF(LEN(I451)=0,"",IF(ISNUMBER(SEARCH(",",I451)),LEN(SUBSTITUTE(I451,",","xx"))-LEN(I451)+1,1))</f>
+        <v/>
+      </c>
       <c r="K451" s="3" t="inlineStr">
         <is>
           <t>%</t>
@@ -39071,9 +39719,16 @@
           <t>升高改善</t>
         </is>
       </c>
-      <c r="M451" s="38" t="n"/>
-      <c r="N451" s="38" t="n"/>
-      <c r="O451" s="16" t="n"/>
+      <c r="M451" s="38" t="n">
+        <v>0</v>
+      </c>
+      <c r="N451" s="38" t="n">
+        <v>1</v>
+      </c>
+      <c r="O451" s="16">
+        <f>IF(AND(N451&lt;0.05,OR(AND(L451="升高改善",M451&gt;0),AND(L451="降低改善",M451&lt;0))),"校正","不校正")</f>
+        <v/>
+      </c>
       <c r="P451" s="3" t="inlineStr">
         <is>
           <t>Fig. 1；PDF第8页，所查看图页未标印刷页码；从上至下第1个Participant One面板；黑色实心方块及实线（Student with ASD）；灰圆及灰虚线为Peer Comparison，不属于本行；纵轴Percentage of Time Engaged。</t>
@@ -39081,17 +39736,17 @@
       </c>
       <c r="Q451" s="3" t="inlineStr">
         <is>
-          <t>GPT</t>
+          <t>Claude</t>
         </is>
       </c>
       <c r="R451" s="35" t="inlineStr">
         <is>
-          <t>待审核</t>
+          <t>Claude补提取</t>
         </is>
       </c>
       <c r="S451" s="3" t="inlineStr">
         <is>
-          <t>待审核：图1被试1和被试2与正文对应的基线均值及干预最小值疑似互换，需先核实被试与曲线的对应关系。</t>
+          <t>Claude补提取（以图为准）：Fig. 1为PDF矢量图，读取黑色实心方块（Student with ASD）的PDF坐标，按各面板0与100位置换算后取整；缺失的观测为学生缺勤（图注）。Participant One面板：基线4点均为0，干预30点均值87.4%、最小值53%。图文不一致：正文写被试1基线1%（0–5%）、干预范围47–100%，与图上Participant Two面板的数值对应，被试1、2在正文中疑似对调。按图（面板标签）取值。</t>
         </is>
       </c>
     </row>
@@ -39213,10 +39868,24 @@
           <t>Baseline（基线期） vs Intervention（干预期）</t>
         </is>
       </c>
-      <c r="G453" s="22" t="n"/>
-      <c r="H453" s="23" t="n"/>
-      <c r="I453" s="22" t="n"/>
-      <c r="J453" s="23" t="n"/>
+      <c r="G453" s="22" t="inlineStr">
+        <is>
+          <t>0,5,0,0</t>
+        </is>
+      </c>
+      <c r="H453" s="23">
+        <f>IF(LEN(G453)=0,"",IF(ISNUMBER(SEARCH(",",G453)),LEN(SUBSTITUTE(G453,",","xx"))-LEN(G453)+1,1))</f>
+        <v/>
+      </c>
+      <c r="I453" s="22" t="inlineStr">
+        <is>
+          <t>88,80,80,100,100,97,100,67,100,100,55,47,87,80,60,70,77,100,100,85,100,100,80,100,100,94,100,70,100,100</t>
+        </is>
+      </c>
+      <c r="J453" s="23">
+        <f>IF(LEN(I453)=0,"",IF(ISNUMBER(SEARCH(",",I453)),LEN(SUBSTITUTE(I453,",","xx"))-LEN(I453)+1,1))</f>
+        <v/>
+      </c>
       <c r="K453" s="8" t="inlineStr">
         <is>
           <t>%</t>
@@ -39227,9 +39896,16 @@
           <t>升高改善</t>
         </is>
       </c>
-      <c r="M453" s="39" t="n"/>
-      <c r="N453" s="39" t="n"/>
-      <c r="O453" s="21" t="n"/>
+      <c r="M453" s="39" t="n">
+        <v>-0.2357022603955159</v>
+      </c>
+      <c r="N453" s="39" t="n">
+        <v>0.6547208460185769</v>
+      </c>
+      <c r="O453" s="21">
+        <f>IF(AND(N453&lt;0.05,OR(AND(L453="升高改善",M453&gt;0),AND(L453="降低改善",M453&lt;0))),"校正","不校正")</f>
+        <v/>
+      </c>
       <c r="P453" s="8" t="inlineStr">
         <is>
           <t>Fig. 1；PDF第8页，所查看图页未标印刷页码；从上至下第2个Participant Two面板；黑色实心方块及实线（Student with ASD）；灰圆及灰虚线为Peer Comparison，不属于本行；纵轴Percentage of Time Engaged。</t>
@@ -39237,17 +39913,17 @@
       </c>
       <c r="Q453" s="8" t="inlineStr">
         <is>
-          <t>GPT</t>
+          <t>Claude</t>
         </is>
       </c>
       <c r="R453" s="24" t="inlineStr">
         <is>
-          <t>待审核</t>
+          <t>Claude补提取</t>
         </is>
       </c>
       <c r="S453" s="8" t="inlineStr">
         <is>
-          <t>待审核：图1被试1和被试2与正文对应的基线均值及干预最小值疑似互换，需先核实被试与曲线的对应关系。</t>
+          <t>Claude补提取（以图为准）：Fig. 1为PDF矢量图，读取黑色实心方块（Student with ASD）的PDF坐标，按各面板0与100位置换算后取整；缺失的观测为学生缺勤（图注）。Participant Two面板：基线4点均值1.25%（0–5%），干预30点均值87.2%、最小值47%。图文不一致：正文写被试2基线0%、干预范围53–100%，与图上Participant One面板对应，疑似对调。按图（面板标签）取值。两名被试同为三年级学生，对调对合并效应量和按年龄段分组没有影响。</t>
         </is>
       </c>
     </row>
@@ -44227,10 +44903,24 @@
           <t>BASELINE（基线期） vs SOCIAL REINFORCEMENT &amp; PROMPTING（社会性强化与提示）</t>
         </is>
       </c>
-      <c r="G513" s="22" t="n"/>
-      <c r="H513" s="23" t="n"/>
-      <c r="I513" s="22" t="n"/>
-      <c r="J513" s="23" t="n"/>
+      <c r="G513" s="22" t="inlineStr">
+        <is>
+          <t>4,4,0,1,1</t>
+        </is>
+      </c>
+      <c r="H513" s="23">
+        <f>IF(LEN(G513)=0,"",IF(ISNUMBER(SEARCH(",",G513)),LEN(SUBSTITUTE(G513,",","xx"))-LEN(G513)+1,1))</f>
+        <v/>
+      </c>
+      <c r="I513" s="22" t="inlineStr">
+        <is>
+          <t>27,16,9,20,17,55,38</t>
+        </is>
+      </c>
+      <c r="J513" s="23">
+        <f>IF(LEN(I513)=0,"",IF(ISNUMBER(SEARCH(",",I513)),LEN(SUBSTITUTE(I513,",","xx"))-LEN(I513)+1,1))</f>
+        <v/>
+      </c>
       <c r="K513" s="18" t="inlineStr">
         <is>
           <t>次/30分钟观察</t>
@@ -44241,9 +44931,16 @@
           <t>升高改善</t>
         </is>
       </c>
-      <c r="M513" s="39" t="n"/>
-      <c r="N513" s="39" t="n"/>
-      <c r="O513" s="21" t="n"/>
+      <c r="M513" s="39" t="n">
+        <v>-0.4472135954999579</v>
+      </c>
+      <c r="N513" s="39" t="n">
+        <v>0.2962698714842864</v>
+      </c>
+      <c r="O513" s="21">
+        <f>IF(AND(N513&lt;0.05,OR(AND(L513="升高改善",M513&gt;0),AND(L513="降低改善",M513&lt;0))),"校正","不校正")</f>
+        <v/>
+      </c>
       <c r="P513" s="18" t="inlineStr">
         <is>
           <t>Figure 2；PDF第11页／印刷第550页；第2面板（Lena，自上而下）；黑色实心圆＝Shadow Therapist；空心圆＝New Therapist，不计入本行</t>
@@ -44251,17 +44948,17 @@
       </c>
       <c r="Q513" s="18" t="inlineStr">
         <is>
-          <t>GPT</t>
+          <t>Claude</t>
         </is>
       </c>
       <c r="R513" s="24" t="inlineStr">
         <is>
-          <t>待审核</t>
+          <t>Claude补提取</t>
         </is>
       </c>
       <c r="S513" s="18" t="inlineStr">
         <is>
-          <t>待审核：基线五个图示点的均值与正文报告不一致，尚不能定位具体错误点，需核实原始基线记录。</t>
+          <t>Claude补提取（以图为准）：从PDF第11页Figure 2内嵌原图（753×557像素，分辨率低，1个单位约1.5像素）检测实心圆，按各面板纵轴刻度换算并扣除0值点的系统偏移（约0.45）；空心圆（New Therapist）不计入。读数精度约±1，落在两个整数中间的点参照正文的均值或范围取整。图文不一致：Lena基线5点为4,4,0,1,1（均值2.0），正文写“0–4次，平均3次”，无法定位，按图取值。干预7点合计182、均值26.0、范围9–55，与正文一致。</t>
         </is>
       </c>
     </row>
@@ -44382,10 +45079,24 @@
           <t>BASELINE（基线期） vs SOCIAL REINFORCEMENT &amp; PROMPTING（社会性强化与提示）</t>
         </is>
       </c>
-      <c r="G515" s="22" t="n"/>
-      <c r="H515" s="23" t="n"/>
-      <c r="I515" s="22" t="n"/>
-      <c r="J515" s="23" t="n"/>
+      <c r="G515" s="22" t="inlineStr">
+        <is>
+          <t>0,0,0,0,0,0,0,0</t>
+        </is>
+      </c>
+      <c r="H515" s="23">
+        <f>IF(LEN(G515)=0,"",IF(ISNUMBER(SEARCH(",",G515)),LEN(SUBSTITUTE(G515,",","xx"))-LEN(G515)+1,1))</f>
+        <v/>
+      </c>
+      <c r="I515" s="22" t="inlineStr">
+        <is>
+          <t>10,2,6,1,18,10,53,48,17,26,18,24</t>
+        </is>
+      </c>
+      <c r="J515" s="23">
+        <f>IF(LEN(I515)=0,"",IF(ISNUMBER(SEARCH(",",I515)),LEN(SUBSTITUTE(I515,",","xx"))-LEN(I515)+1,1))</f>
+        <v/>
+      </c>
       <c r="K515" s="18" t="inlineStr">
         <is>
           <t>次/30分钟观察</t>
@@ -44396,9 +45107,16 @@
           <t>升高改善</t>
         </is>
       </c>
-      <c r="M515" s="39" t="n"/>
-      <c r="N515" s="39" t="n"/>
-      <c r="O515" s="21" t="n"/>
+      <c r="M515" s="39" t="n">
+        <v>0</v>
+      </c>
+      <c r="N515" s="39" t="n">
+        <v>1</v>
+      </c>
+      <c r="O515" s="21">
+        <f>IF(AND(N515&lt;0.05,OR(AND(L515="升高改善",M515&gt;0),AND(L515="降低改善",M515&lt;0))),"校正","不校正")</f>
+        <v/>
+      </c>
       <c r="P515" s="18" t="inlineStr">
         <is>
           <t>Figure 2；PDF第11页／印刷第550页；第3面板（Andrew，自上而下）；黑色实心圆＝Shadow Therapist；空心圆＝New Therapist，不计入本行</t>
@@ -44406,17 +45124,17 @@
       </c>
       <c r="Q515" s="18" t="inlineStr">
         <is>
-          <t>GPT</t>
+          <t>Claude</t>
         </is>
       </c>
       <c r="R515" s="24" t="inlineStr">
         <is>
-          <t>待审核</t>
+          <t>Claude补提取</t>
         </is>
       </c>
       <c r="S515" s="18" t="inlineStr">
         <is>
-          <t>待审核：干预图示最小值与正文报告的下限不一致，尚不能确定差异来源，需核实对应观察点。</t>
+          <t>Claude补提取（以图为准）：从PDF第11页Figure 2内嵌原图（753×557像素，分辨率低，1个单位约1.5像素）检测实心圆，按各面板纵轴刻度换算并扣除0值点的系统偏移（约0.45）；空心圆（New Therapist）不计入。读数精度约±1，落在两个整数中间的点参照正文的均值或范围取整。图文不一致：Andrew干预第4点（第12次）图上约为1，低于正文报告的下限2（正文范围2–53）；干预12点均值19.4，正文约20。按图取值。</t>
         </is>
       </c>
     </row>
@@ -44538,10 +45256,24 @@
           <t>BASELINE（基线期） vs SOCIAL REINFORCEMENT &amp; PROMPTING（社会性强化与提示）</t>
         </is>
       </c>
-      <c r="G517" s="22" t="n"/>
-      <c r="H517" s="23" t="n"/>
-      <c r="I517" s="22" t="n"/>
-      <c r="J517" s="23" t="n"/>
+      <c r="G517" s="22" t="inlineStr">
+        <is>
+          <t>0,0,0,0,0,0,0,0,0,0</t>
+        </is>
+      </c>
+      <c r="H517" s="23">
+        <f>IF(LEN(G517)=0,"",IF(ISNUMBER(SEARCH(",",G517)),LEN(SUBSTITUTE(G517,",","xx"))-LEN(G517)+1,1))</f>
+        <v/>
+      </c>
+      <c r="I517" s="22" t="inlineStr">
+        <is>
+          <t>4,6,10,8,16,20,14,18,20,17,23</t>
+        </is>
+      </c>
+      <c r="J517" s="23">
+        <f>IF(LEN(I517)=0,"",IF(ISNUMBER(SEARCH(",",I517)),LEN(SUBSTITUTE(I517,",","xx"))-LEN(I517)+1,1))</f>
+        <v/>
+      </c>
       <c r="K517" s="18" t="inlineStr">
         <is>
           <t>次/30分钟观察</t>
@@ -44552,9 +45284,16 @@
           <t>升高改善</t>
         </is>
       </c>
-      <c r="M517" s="39" t="n"/>
-      <c r="N517" s="39" t="n"/>
-      <c r="O517" s="21" t="n"/>
+      <c r="M517" s="39" t="n">
+        <v>0</v>
+      </c>
+      <c r="N517" s="39" t="n">
+        <v>1</v>
+      </c>
+      <c r="O517" s="21">
+        <f>IF(AND(N517&lt;0.05,OR(AND(L517="升高改善",M517&gt;0),AND(L517="降低改善",M517&lt;0))),"校正","不校正")</f>
+        <v/>
+      </c>
       <c r="P517" s="18" t="inlineStr">
         <is>
           <t>Figure 2；PDF第11页／印刷第550页；第4面板（Cory，自上而下）；黑色实心圆＝Shadow Therapist；空心圆＝New Therapist，不计入本行</t>
@@ -44562,17 +45301,17 @@
       </c>
       <c r="Q517" s="18" t="inlineStr">
         <is>
-          <t>GPT</t>
+          <t>Claude</t>
         </is>
       </c>
       <c r="R517" s="24" t="inlineStr">
         <is>
-          <t>待审核</t>
+          <t>Claude补提取</t>
         </is>
       </c>
       <c r="S517" s="18" t="inlineStr">
         <is>
-          <t>待审核：干预图示点的均值与正文报告不一致，尚不能判断是读图偏差还是文字误差，需核实干预序列。</t>
+          <t>Claude补提取（以图为准）：从PDF第11页Figure 2内嵌原图（753×557像素，分辨率低，1个单位约1.5像素）检测实心圆，按各面板纵轴刻度换算并扣除0值点的系统偏移（约0.45）；空心圆（New Therapist）不计入。读数精度约±1，落在两个整数中间的点参照正文的均值或范围取整。Cory干预11点均值14.2、范围4–23，与正文（平均14，4–23）一致；最后一点图上约22.4，按正文上限取23。原先所说的均值不一致按此读数不存在。</t>
         </is>
       </c>
     </row>
@@ -45849,7 +46588,7 @@
       </c>
       <c r="S532" s="18" t="inlineStr">
         <is>
-          <t>待审核：教师介入阶段第12个观察点的图示值超出正文报告上限，图文范围冲突，需核实对应数据。</t>
+          <t>【Claude第二轮：未提取】图为扫描件，数据点小而密集、贴近横轴，按用户要求“实在模糊、看不清就空着”，本行不填。　原备注：待审核：教师介入阶段第12个观察点的图示值超出正文报告上限，图文范围冲突，需核实对应数据。</t>
         </is>
       </c>
     </row>
@@ -45918,7 +46657,7 @@
       </c>
       <c r="S533" s="18" t="inlineStr">
         <is>
-          <t>待审核：教师介入阶段第15、18个观察点的图示值超出正文报告上限，需核实两点后确认比较序列。</t>
+          <t>【Claude第二轮：未提取】图为扫描件，数据点小而密集、贴近横轴，按用户要求“实在模糊、看不清就空着”，本行不填。　原备注：待审核：教师介入阶段第15、18个观察点的图示值超出正文报告上限，需核实两点后确认比较序列。</t>
         </is>
       </c>
     </row>
@@ -45987,7 +46726,7 @@
       </c>
       <c r="S534" s="18" t="inlineStr">
         <is>
-          <t>待审核：教师介入阶段第4个观察点的图示值超出正文报告上限，图文范围冲突，需核实对应数据。</t>
+          <t>【Claude第二轮：未提取】图为扫描件，数据点小而密集、贴近横轴，按用户要求“实在模糊、看不清就空着”，本行不填。　原备注：待审核：教师介入阶段第4个观察点的图示值超出正文报告上限，图文范围冲突，需核实对应数据。</t>
         </is>
       </c>
     </row>
@@ -47752,10 +48491,24 @@
           <t>baseline（基线期） vs intervention（干预期）</t>
         </is>
       </c>
-      <c r="G555" s="22" t="n"/>
-      <c r="H555" s="23" t="n"/>
-      <c r="I555" s="22" t="n"/>
-      <c r="J555" s="23" t="n"/>
+      <c r="G555" s="22" t="inlineStr">
+        <is>
+          <t>8,1,2,6,5,1,1,3,3</t>
+        </is>
+      </c>
+      <c r="H555" s="23">
+        <f>IF(LEN(G555)=0,"",IF(ISNUMBER(SEARCH(",",G555)),LEN(SUBSTITUTE(G555,",","xx"))-LEN(G555)+1,1))</f>
+        <v/>
+      </c>
+      <c r="I555" s="22" t="inlineStr">
+        <is>
+          <t>22,27,22,15,24,11,51,6,29,20,33</t>
+        </is>
+      </c>
+      <c r="J555" s="23">
+        <f>IF(LEN(I555)=0,"",IF(ISNUMBER(SEARCH(",",I555)),LEN(SUBSTITUTE(I555,",","xx"))-LEN(I555)+1,1))</f>
+        <v/>
+      </c>
       <c r="K555" s="18" t="inlineStr">
         <is>
           <t>次/10分钟</t>
@@ -47766,9 +48519,16 @@
           <t>升高改善</t>
         </is>
       </c>
-      <c r="M555" s="39" t="n"/>
-      <c r="N555" s="39" t="n"/>
-      <c r="O555" s="21" t="n"/>
+      <c r="M555" s="39" t="n">
+        <v>-0.1767766952966369</v>
+      </c>
+      <c r="N555" s="39" t="n">
+        <v>0.5208480313753976</v>
+      </c>
+      <c r="O555" s="21">
+        <f>IF(AND(N555&lt;0.05,OR(AND(L555="升高改善",M555&gt;0),AND(L555="降低改善",M555&lt;0))),"校正","不校正")</f>
+        <v/>
+      </c>
       <c r="P555" s="18" t="inlineStr">
         <is>
           <t>Figure 2；PDF第18页／稿件印刷Page 18（期刊页码未标）；下面板（Brian）；黑色实心圆、实线连接；阶段名称取自Figure 2图注</t>
@@ -47776,17 +48536,17 @@
       </c>
       <c r="Q555" s="18" t="inlineStr">
         <is>
-          <t>GPT</t>
+          <t>Claude</t>
         </is>
       </c>
       <c r="R555" s="24" t="inlineStr">
         <is>
-          <t>待审核</t>
+          <t>Claude补提取</t>
         </is>
       </c>
       <c r="S555" s="18" t="inlineStr">
         <is>
-          <t>待审核：基线9个图示点的均值与正文报告不符，且准确会话号尚未确认，需同时核实基线读值和时间对应。</t>
+          <t>Claude补提取（以图为准）：从PDF第18页内嵌图像逐像素检测Brian面板圆点，按纵轴刻度标签换算（同D0552）；基线第3、4次和第5、6次两两相邻重叠，按合并重心和形状拆分为1,2和6,5。会话号对应不影响Tau-U。图文不一致：基线9点均值3.33，正文报告3.8（范围1–8与图一致），无法定位，按图取值。干预11点均值23.6、范围6–51，与正文一致。</t>
         </is>
       </c>
     </row>
@@ -51125,10 +51885,24 @@
           <t>基线期 vs 干预期</t>
         </is>
       </c>
-      <c r="G596" s="22" t="n"/>
-      <c r="H596" s="23" t="n"/>
-      <c r="I596" s="22" t="n"/>
-      <c r="J596" s="23" t="n"/>
+      <c r="G596" s="22" t="inlineStr">
+        <is>
+          <t>0,1,0,2,1,0,1</t>
+        </is>
+      </c>
+      <c r="H596" s="23">
+        <f>IF(LEN(G596)=0,"",IF(ISNUMBER(SEARCH(",",G596)),LEN(SUBSTITUTE(G596,",","xx"))-LEN(G596)+1,1))</f>
+        <v/>
+      </c>
+      <c r="I596" s="22" t="inlineStr">
+        <is>
+          <t>3,5,6,7,16,8,23,10,14,20,18,18,20,19,15,19</t>
+        </is>
+      </c>
+      <c r="J596" s="23">
+        <f>IF(LEN(I596)=0,"",IF(ISNUMBER(SEARCH(",",I596)),LEN(SUBSTITUTE(I596,",","xx"))-LEN(I596)+1,1))</f>
+        <v/>
+      </c>
       <c r="K596" s="18" t="inlineStr">
         <is>
           <t>次</t>
@@ -51139,9 +51913,16 @@
           <t>升高改善</t>
         </is>
       </c>
-      <c r="M596" s="39" t="n"/>
-      <c r="N596" s="39" t="n"/>
-      <c r="O596" s="21" t="n"/>
+      <c r="M596" s="39" t="n">
+        <v>0.1690308509457033</v>
+      </c>
+      <c r="N596" s="39" t="n">
+        <v>0.621873424330741</v>
+      </c>
+      <c r="O596" s="21">
+        <f>IF(AND(N596&lt;0.05,OR(AND(L596="升高改善",M596&gt;0),AND(L596="降低改善",M596&lt;0))),"校正","不校正")</f>
+        <v/>
+      </c>
       <c r="P596" s="18" t="inlineStr">
         <is>
           <t>图1“3名被试社交发起与回应行为频次变化折线图”；PDF第5页，印刷页61；从上至下第3个被试小翰面板；实心圆（发起次数）；纵轴行为次数，横轴观察次数；基线期与干预期。</t>
@@ -51149,17 +51930,17 @@
       </c>
       <c r="Q596" s="18" t="inlineStr">
         <is>
-          <t>GPT</t>
+          <t>Claude</t>
         </is>
       </c>
       <c r="R596" s="24" t="inlineStr">
         <is>
-          <t>待审核</t>
+          <t>Claude补提取</t>
         </is>
       </c>
       <c r="S596" s="18" t="inlineStr">
         <is>
-          <t>待审核：干预图连续显示16个观察点，正文却称缺席2次，无法确定缺失会话与图示点的对应关系。</t>
+          <t>Claude补提取（以图为准）：从PDF第5页内嵌原图（2362×3668像素）逐像素检测圆点（发起）和方块（回应），按纵轴刻度（每单位约11.9像素）换算。基线7点：发起0,1,0,2,1,0,1（均值0.71），回应2,2,1,1,2,1,1（均值1.43），均落在正文报告的基线均值范围内（发起0.67–1，回应1.33–1.60）；基线两条线多处重叠，第7次两个符号重合于1，依据正文均值范围确定。干预期图上16点，合计221，221÷16=13.81，与正文均值13.81完全一致，说明作者也按16点计算；正文“小翰缺席2次”与数据点数的矛盾属叙述问题，按图取16点。</t>
         </is>
       </c>
     </row>
@@ -51194,10 +51975,24 @@
           <t>基线期 vs 维持期</t>
         </is>
       </c>
-      <c r="G597" s="22" t="n"/>
-      <c r="H597" s="23" t="n"/>
-      <c r="I597" s="22" t="n"/>
-      <c r="J597" s="23" t="n"/>
+      <c r="G597" s="22" t="inlineStr">
+        <is>
+          <t>0,1,0,2,1,0,1</t>
+        </is>
+      </c>
+      <c r="H597" s="23">
+        <f>IF(LEN(G597)=0,"",IF(ISNUMBER(SEARCH(",",G597)),LEN(SUBSTITUTE(G597,",","xx"))-LEN(G597)+1,1))</f>
+        <v/>
+      </c>
+      <c r="I597" s="22" t="inlineStr">
+        <is>
+          <t>16,18,15,16,17</t>
+        </is>
+      </c>
+      <c r="J597" s="23">
+        <f>IF(LEN(I597)=0,"",IF(ISNUMBER(SEARCH(",",I597)),LEN(SUBSTITUTE(I597,",","xx"))-LEN(I597)+1,1))</f>
+        <v/>
+      </c>
       <c r="K597" s="18" t="inlineStr">
         <is>
           <t>次</t>
@@ -51208,9 +52003,16 @@
           <t>升高改善</t>
         </is>
       </c>
-      <c r="M597" s="39" t="n"/>
-      <c r="N597" s="39" t="n"/>
-      <c r="O597" s="21" t="n"/>
+      <c r="M597" s="39" t="n">
+        <v>0.1690308509457033</v>
+      </c>
+      <c r="N597" s="39" t="n">
+        <v>0.621873424330741</v>
+      </c>
+      <c r="O597" s="21">
+        <f>IF(AND(N597&lt;0.05,OR(AND(L597="升高改善",M597&gt;0),AND(L597="降低改善",M597&lt;0))),"校正","不校正")</f>
+        <v/>
+      </c>
       <c r="P597" s="18" t="inlineStr">
         <is>
           <t>图1“3名被试社交发起与回应行为频次变化折线图”；PDF第5页，印刷页61；从上至下第3个被试小翰面板；实心圆（发起次数）；纵轴行为次数，横轴观察次数；右侧维持期。</t>
@@ -51218,17 +52020,17 @@
       </c>
       <c r="Q597" s="18" t="inlineStr">
         <is>
-          <t>GPT</t>
+          <t>Claude</t>
         </is>
       </c>
       <c r="R597" s="24" t="inlineStr">
         <is>
-          <t>待审核</t>
+          <t>Claude补提取</t>
         </is>
       </c>
       <c r="S597" s="18" t="inlineStr">
         <is>
-          <t>待审核：维持阶段五个图示点的均值与正文报告不一致，尚无法定位具体错误点，需核实完整维持序列。</t>
+          <t>Claude补提取（以图为准）：从PDF第5页内嵌原图（2362×3668像素）逐像素检测圆点（发起）和方块（回应），按纵轴刻度（每单位约11.9像素）换算。基线7点：发起0,1,0,2,1,0,1（均值0.71），回应2,2,1,1,2,1,1（均值1.43），均落在正文报告的基线均值范围内（发起0.67–1，回应1.33–1.60）；基线两条线多处重叠，第7次两个符号重合于1，依据正文均值范围确定。图文不一致：维持期图上5点均值16.4，正文报告18.4，无法定位具体哪个点，按图取值。</t>
         </is>
       </c>
     </row>
@@ -51263,10 +52065,24 @@
           <t>基线期 vs 干预期</t>
         </is>
       </c>
-      <c r="G598" s="22" t="n"/>
-      <c r="H598" s="23" t="n"/>
-      <c r="I598" s="22" t="n"/>
-      <c r="J598" s="23" t="n"/>
+      <c r="G598" s="22" t="inlineStr">
+        <is>
+          <t>2,2,1,1,2,1,1</t>
+        </is>
+      </c>
+      <c r="H598" s="23">
+        <f>IF(LEN(G598)=0,"",IF(ISNUMBER(SEARCH(",",G598)),LEN(SUBSTITUTE(G598,",","xx"))-LEN(G598)+1,1))</f>
+        <v/>
+      </c>
+      <c r="I598" s="22" t="inlineStr">
+        <is>
+          <t>25,21,33,28,35,35,56,39,51,37,57,61,60,55,66,58</t>
+        </is>
+      </c>
+      <c r="J598" s="23">
+        <f>IF(LEN(I598)=0,"",IF(ISNUMBER(SEARCH(",",I598)),LEN(SUBSTITUTE(I598,",","xx"))-LEN(I598)+1,1))</f>
+        <v/>
+      </c>
       <c r="K598" s="18" t="inlineStr">
         <is>
           <t>次</t>
@@ -51277,9 +52093,16 @@
           <t>升高改善</t>
         </is>
       </c>
-      <c r="M598" s="39" t="n"/>
-      <c r="N598" s="39" t="n"/>
-      <c r="O598" s="21" t="n"/>
+      <c r="M598" s="39" t="n">
+        <v>-0.5039526306789697</v>
+      </c>
+      <c r="N598" s="39" t="n">
+        <v>0.1572992070502852</v>
+      </c>
+      <c r="O598" s="21">
+        <f>IF(AND(N598&lt;0.05,OR(AND(L598="升高改善",M598&gt;0),AND(L598="降低改善",M598&lt;0))),"校正","不校正")</f>
+        <v/>
+      </c>
       <c r="P598" s="18" t="inlineStr">
         <is>
           <t>图1“3名被试社交发起与回应行为频次变化折线图”；PDF第5页，印刷页61；从上至下第3个被试小翰面板；实心方块（回应次数）；纵轴行为次数，横轴观察次数；基线期与干预期。</t>
@@ -51287,17 +52110,17 @@
       </c>
       <c r="Q598" s="18" t="inlineStr">
         <is>
-          <t>GPT</t>
+          <t>Claude</t>
         </is>
       </c>
       <c r="R598" s="24" t="inlineStr">
         <is>
-          <t>待审核</t>
+          <t>Claude补提取</t>
         </is>
       </c>
       <c r="S598" s="18" t="inlineStr">
         <is>
-          <t>待审核：干预图连续显示16个观察点，正文却称缺席2次，无法确定缺失会话与图示点的对应关系。</t>
+          <t>Claude补提取（以图为准）：从PDF第5页内嵌原图（2362×3668像素）逐像素检测圆点（发起）和方块（回应），按纵轴刻度（每单位约11.9像素）换算。基线7点：发起0,1,0,2,1,0,1（均值0.71），回应2,2,1,1,2,1,1（均值1.43），均落在正文报告的基线均值范围内（发起0.67–1，回应1.33–1.60）；基线两条线多处重叠，第7次两个符号重合于1，依据正文均值范围确定。干预期图上16点，合计717，717÷16=44.81，与正文均值44.81完全一致；正文“缺席2次”与点数的矛盾同D0595，按图取16点。</t>
         </is>
       </c>
     </row>
@@ -51332,10 +52155,24 @@
           <t>基线期 vs 维持期</t>
         </is>
       </c>
-      <c r="G599" s="22" t="n"/>
-      <c r="H599" s="23" t="n"/>
-      <c r="I599" s="22" t="n"/>
-      <c r="J599" s="23" t="n"/>
+      <c r="G599" s="22" t="inlineStr">
+        <is>
+          <t>2,2,1,1,2,1,1</t>
+        </is>
+      </c>
+      <c r="H599" s="23">
+        <f>IF(LEN(G599)=0,"",IF(ISNUMBER(SEARCH(",",G599)),LEN(SUBSTITUTE(G599,",","xx"))-LEN(G599)+1,1))</f>
+        <v/>
+      </c>
+      <c r="I599" s="22" t="inlineStr">
+        <is>
+          <t>33,40,35,38,41</t>
+        </is>
+      </c>
+      <c r="J599" s="23">
+        <f>IF(LEN(I599)=0,"",IF(ISNUMBER(SEARCH(",",I599)),LEN(SUBSTITUTE(I599,",","xx"))-LEN(I599)+1,1))</f>
+        <v/>
+      </c>
       <c r="K599" s="18" t="inlineStr">
         <is>
           <t>次</t>
@@ -51346,9 +52183,16 @@
           <t>升高改善</t>
         </is>
       </c>
-      <c r="M599" s="39" t="n"/>
-      <c r="N599" s="39" t="n"/>
-      <c r="O599" s="21" t="n"/>
+      <c r="M599" s="39" t="n">
+        <v>-0.5039526306789697</v>
+      </c>
+      <c r="N599" s="39" t="n">
+        <v>0.1572992070502852</v>
+      </c>
+      <c r="O599" s="21">
+        <f>IF(AND(N599&lt;0.05,OR(AND(L599="升高改善",M599&gt;0),AND(L599="降低改善",M599&lt;0))),"校正","不校正")</f>
+        <v/>
+      </c>
       <c r="P599" s="18" t="inlineStr">
         <is>
           <t>图1“3名被试社交发起与回应行为频次变化折线图”；PDF第5页，印刷页61；从上至下第3个被试小翰面板；实心方块（回应次数）；纵轴行为次数，横轴观察次数；右侧维持期。</t>
@@ -51356,17 +52200,17 @@
       </c>
       <c r="Q599" s="18" t="inlineStr">
         <is>
-          <t>GPT</t>
+          <t>Claude</t>
         </is>
       </c>
       <c r="R599" s="24" t="inlineStr">
         <is>
-          <t>待审核</t>
+          <t>Claude补提取</t>
         </is>
       </c>
       <c r="S599" s="18" t="inlineStr">
         <is>
-          <t>待审核：维持阶段五个图示点的均值与正文报告不一致，尚无法定位具体错误点，需核实完整维持序列。</t>
+          <t>Claude补提取（以图为准）：从PDF第5页内嵌原图（2362×3668像素）逐像素检测圆点（发起）和方块（回应），按纵轴刻度（每单位约11.9像素）换算。基线7点：发起0,1,0,2,1,0,1（均值0.71），回应2,2,1,1,2,1,1（均值1.43），均落在正文报告的基线均值范围内（发起0.67–1，回应1.33–1.60）；基线两条线多处重叠，第7次两个符号重合于1，依据正文均值范围确定。图文不一致：维持期图上5点均值37.4，正文报告38，无法定位具体哪个点，按图取值。</t>
         </is>
       </c>
     </row>
@@ -51385,7 +52229,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B9"/>
+  <dimension ref="A1:B17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -51496,6 +52340,90 @@
         </is>
       </c>
     </row>
+    <row r="10">
+      <c r="A10" s="43" t="inlineStr"/>
+      <c r="B10" s="43" t="inlineStr"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="43" t="inlineStr">
+        <is>
+          <t>第二轮补提取（以图为准）</t>
+        </is>
+      </c>
+      <c r="B11" s="43" t="inlineStr"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="43" t="inlineStr">
+        <is>
+          <t>依据</t>
+        </is>
+      </c>
+      <c r="B12" s="43" t="inlineStr">
+        <is>
+          <t>用户确定：图文数值不一致时以图为准；点数、阶段归属、被试对应不清时，按图上的数据点和阶段线取值；实在模糊、看不清的不提取。</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="43" t="inlineStr">
+        <is>
+          <t>补提取范围</t>
+        </is>
+      </c>
+      <c r="B13" s="43" t="inlineStr">
+        <is>
+          <t>40行：张晓敏2026 4行、013-A 2行、009-A 3行、011-A 5行、021-A 1行、025-A 2行、030-A 1行、035-A 2行、039-A 3行、036-A 4行、044-A 7行、046-A 2行、22 Mason 2014 Brian 1行、09 Gena 2006 3行。每行备注写明读图方法、正文报告的数值和差异。</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="43" t="inlineStr">
+        <is>
+          <t>未提取</t>
+        </is>
+      </c>
+      <c r="B14" s="43" t="inlineStr">
+        <is>
+          <t>17 Kern 2006的D0531–D0533：扫描图，数据点小而密集，按“看不清就空着”不填，备注已注明。比较方式待作者确定的22行（022-A、03 Blair、24 Morrison、017-A）本轮未动。</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="43" t="inlineStr">
+        <is>
+          <t>改动比较类型的行</t>
+        </is>
+      </c>
+      <c r="B15" s="43" t="inlineStr">
+        <is>
+          <t>036-A的D0356、D0357、D0358原比较类型为“待审核”，按图上阶段线改为“干预”（Baseline vs VP Intervention）；维持期数值写在备注中，如需维持效应可另加行。</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="43" t="inlineStr">
+        <is>
+          <t>对GPT已填行的提示</t>
+        </is>
+      </c>
+      <c r="B16" s="43" t="inlineStr">
+        <is>
+          <t>D0321、D0323（035-A Emmett发起）：基线第4次按符号形状判断可能应为3而非2，只在备注中提示，数值未改。</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="43" t="inlineStr">
+        <is>
+          <t>读图方法</t>
+        </is>
+      </c>
+      <c r="B17" s="43" t="inlineStr">
+        <is>
+          <t>矢量图（011-A、025-A、036-A、039-A、046-A）直接读取PDF中数据符号的坐标；位图按灰度识别符号并逐像素取中心，用刻度线或刻度标签换算；重叠或被遮挡的符号用可见边缘加符号半径推算。09 Gena 2006原图分辨率低（1个单位约1.5像素），落在两个整数中间的点参照正文均值或范围取整。</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Mark the three Kern 2006 rows (Ben, Phillip, Lucas) as not included
Author decision: the scanned figure is too blurry to extract, so
D0531-D0533 stay blank and are marked 不纳入. D0530 (Eric) is unchanged.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_015FN8gfsh3be5UpV8911V5L
</commit_message>
<xml_diff>
--- a/Tau-U计算前准备数据_完整版_中英对照_网格版_Claude补提取版.xlsx
+++ b/Tau-U计算前准备数据_完整版_中英对照_网格版_Claude补提取版.xlsx
@@ -46583,12 +46583,12 @@
       </c>
       <c r="R532" s="24" t="inlineStr">
         <is>
-          <t>待审核</t>
+          <t>不纳入</t>
         </is>
       </c>
       <c r="S532" s="18" t="inlineStr">
         <is>
-          <t>【Claude第二轮：未提取】图为扫描件，数据点小而密集、贴近横轴，按用户要求“实在模糊、看不清就空着”，本行不填。　原备注：待审核：教师介入阶段第12个观察点的图示值超出正文报告上限，图文范围冲突，需核实对应数据。</t>
+          <t>【不纳入】作者决定：17 Kern 2006的Figure 1为扫描图，数据点模糊难以提取，Ben、Phillip、Lucas三行不纳入Tau-U计算。　【Claude第二轮：未提取】图为扫描件，数据点小而密集、贴近横轴，按用户要求“实在模糊、看不清就空着”，本行不填。　原备注：待审核：教师介入阶段第12个观察点的图示值超出正文报告上限，图文范围冲突，需核实对应数据。</t>
         </is>
       </c>
     </row>
@@ -46652,12 +46652,12 @@
       </c>
       <c r="R533" s="24" t="inlineStr">
         <is>
-          <t>待审核</t>
+          <t>不纳入</t>
         </is>
       </c>
       <c r="S533" s="18" t="inlineStr">
         <is>
-          <t>【Claude第二轮：未提取】图为扫描件，数据点小而密集、贴近横轴，按用户要求“实在模糊、看不清就空着”，本行不填。　原备注：待审核：教师介入阶段第15、18个观察点的图示值超出正文报告上限，需核实两点后确认比较序列。</t>
+          <t>【不纳入】作者决定：17 Kern 2006的Figure 1为扫描图，数据点模糊难以提取，Ben、Phillip、Lucas三行不纳入Tau-U计算。　【Claude第二轮：未提取】图为扫描件，数据点小而密集、贴近横轴，按用户要求“实在模糊、看不清就空着”，本行不填。　原备注：待审核：教师介入阶段第15、18个观察点的图示值超出正文报告上限，需核实两点后确认比较序列。</t>
         </is>
       </c>
     </row>
@@ -46721,12 +46721,12 @@
       </c>
       <c r="R534" s="24" t="inlineStr">
         <is>
-          <t>待审核</t>
+          <t>不纳入</t>
         </is>
       </c>
       <c r="S534" s="18" t="inlineStr">
         <is>
-          <t>【Claude第二轮：未提取】图为扫描件，数据点小而密集、贴近横轴，按用户要求“实在模糊、看不清就空着”，本行不填。　原备注：待审核：教师介入阶段第4个观察点的图示值超出正文报告上限，图文范围冲突，需核实对应数据。</t>
+          <t>【不纳入】作者决定：17 Kern 2006的Figure 1为扫描图，数据点模糊难以提取，Ben、Phillip、Lucas三行不纳入Tau-U计算。　【Claude第二轮：未提取】图为扫描件，数据点小而密集、贴近横轴，按用户要求“实在模糊、看不清就空着”，本行不填。　原备注：待审核：教师介入阶段第4个观察点的图示值超出正文报告上限，图文范围冲突，需核实对应数据。</t>
         </is>
       </c>
     </row>
@@ -52229,7 +52229,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B17"/>
+  <dimension ref="A1:B18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -52424,6 +52424,18 @@
         </is>
       </c>
     </row>
+    <row r="18">
+      <c r="A18" s="43" t="inlineStr">
+        <is>
+          <t>Kern不纳入</t>
+        </is>
+      </c>
+      <c r="B18" s="43" t="inlineStr">
+        <is>
+          <t>作者决定：17 Kern 2006的D0531（Ben）、D0532（Phillip）、D0533（Lucas）三行因扫描图模糊不纳入，审核状态改为“不纳入”，数值保持空白。D0530（Eric，GPT已填）未改动。</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Set the three Kern 2006 rows back to pending review
Author decision: D0531-D0533 are marked 待审核 rather than 不纳入;
values stay blank and the note explains the blurry scanned figure.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_015FN8gfsh3be5UpV8911V5L
</commit_message>
<xml_diff>
--- a/Tau-U计算前准备数据_完整版_中英对照_网格版_Claude补提取版.xlsx
+++ b/Tau-U计算前准备数据_完整版_中英对照_网格版_Claude补提取版.xlsx
@@ -46583,12 +46583,12 @@
       </c>
       <c r="R532" s="24" t="inlineStr">
         <is>
-          <t>不纳入</t>
+          <t>待审核</t>
         </is>
       </c>
       <c r="S532" s="18" t="inlineStr">
         <is>
-          <t>【不纳入】作者决定：17 Kern 2006的Figure 1为扫描图，数据点模糊难以提取，Ben、Phillip、Lucas三行不纳入Tau-U计算。　【Claude第二轮：未提取】图为扫描件，数据点小而密集、贴近横轴，按用户要求“实在模糊、看不清就空着”，本行不填。　原备注：待审核：教师介入阶段第12个观察点的图示值超出正文报告上限，图文范围冲突，需核实对应数据。</t>
+          <t>【待审核】17 Kern 2006的Figure 1为扫描图，数据点模糊难以提取，Ben、Phillip、Lucas三行暂不提取。　【Claude第二轮：未提取】图为扫描件，数据点小而密集、贴近横轴，按用户要求“实在模糊、看不清就空着”，本行不填。　原备注：待审核：教师介入阶段第12个观察点的图示值超出正文报告上限，图文范围冲突，需核实对应数据。</t>
         </is>
       </c>
     </row>
@@ -46652,12 +46652,12 @@
       </c>
       <c r="R533" s="24" t="inlineStr">
         <is>
-          <t>不纳入</t>
+          <t>待审核</t>
         </is>
       </c>
       <c r="S533" s="18" t="inlineStr">
         <is>
-          <t>【不纳入】作者决定：17 Kern 2006的Figure 1为扫描图，数据点模糊难以提取，Ben、Phillip、Lucas三行不纳入Tau-U计算。　【Claude第二轮：未提取】图为扫描件，数据点小而密集、贴近横轴，按用户要求“实在模糊、看不清就空着”，本行不填。　原备注：待审核：教师介入阶段第15、18个观察点的图示值超出正文报告上限，需核实两点后确认比较序列。</t>
+          <t>【待审核】17 Kern 2006的Figure 1为扫描图，数据点模糊难以提取，Ben、Phillip、Lucas三行暂不提取。　【Claude第二轮：未提取】图为扫描件，数据点小而密集、贴近横轴，按用户要求“实在模糊、看不清就空着”，本行不填。　原备注：待审核：教师介入阶段第15、18个观察点的图示值超出正文报告上限，需核实两点后确认比较序列。</t>
         </is>
       </c>
     </row>
@@ -46721,12 +46721,12 @@
       </c>
       <c r="R534" s="24" t="inlineStr">
         <is>
-          <t>不纳入</t>
+          <t>待审核</t>
         </is>
       </c>
       <c r="S534" s="18" t="inlineStr">
         <is>
-          <t>【不纳入】作者决定：17 Kern 2006的Figure 1为扫描图，数据点模糊难以提取，Ben、Phillip、Lucas三行不纳入Tau-U计算。　【Claude第二轮：未提取】图为扫描件，数据点小而密集、贴近横轴，按用户要求“实在模糊、看不清就空着”，本行不填。　原备注：待审核：教师介入阶段第4个观察点的图示值超出正文报告上限，图文范围冲突，需核实对应数据。</t>
+          <t>【待审核】17 Kern 2006的Figure 1为扫描图，数据点模糊难以提取，Ben、Phillip、Lucas三行暂不提取。　【Claude第二轮：未提取】图为扫描件，数据点小而密集、贴近横轴，按用户要求“实在模糊、看不清就空着”，本行不填。　原备注：待审核：教师介入阶段第4个观察点的图示值超出正文报告上限，图文范围冲突，需核实对应数据。</t>
         </is>
       </c>
     </row>
@@ -52427,12 +52427,12 @@
     <row r="18">
       <c r="A18" s="43" t="inlineStr">
         <is>
-          <t>Kern不纳入</t>
+          <t>Kern待审核</t>
         </is>
       </c>
       <c r="B18" s="43" t="inlineStr">
         <is>
-          <t>作者决定：17 Kern 2006的D0531（Ben）、D0532（Phillip）、D0533（Lucas）三行因扫描图模糊不纳入，审核状态改为“不纳入”，数值保持空白。D0530（Eric，GPT已填）未改动。</t>
+          <t>17 Kern 2006的D0531（Ben）、D0532（Phillip）、D0533（Lucas）三行因扫描图模糊暂不提取，审核状态为“待审核”，数值保持空白。D0530（Eric，GPT已填）未改动。</t>
         </is>
       </c>
     </row>

</xml_diff>